<commit_message>
Glossary terms at analyser execution
</commit_message>
<xml_diff>
--- a/LATEST_SCHEMA/schema_azure_mssql_dbo.xlsx
+++ b/LATEST_SCHEMA/schema_azure_mssql_dbo.xlsx
@@ -826,7 +826,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -965,7 +965,11 @@
           <t>Procurement headers including approver employee relationship.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.PurchaseOrder, RetailDomainGlossary.OrderStatus</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>{"concept_counts":{"entity.status":1,"identifier.foreign_key":4,"temporal.created_at":1,"temporal.date_only":2,"temporal.updated_at":1},"low_confidence_columns":[]}</t>
@@ -1493,10 +1497,14 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Unique identifier for purchase orders in the retail operations system.</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
+          <t>Unique identifier for purchase orders in the system.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.PurchaseOrder</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -1572,10 +1580,14 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>References the unique identifier of the supplier associated with a purchase order, linking to the `suppliers.supplier_id` column.</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
+          <t>Identifies the supplier associated with a purchase order, referencing the `supplier_id` column in the `suppliers` table.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SupplierCode</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -1738,10 +1750,14 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Indicates the current state of a purchase order, such as 'Ordered' or 'Received', using predefined category values.</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr"/>
+          <t>Indicates the current state of a purchase order (e.g., "Ordered," "Received") as a non-null categorical value.</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.OrderStatus</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>entity.status</t>
@@ -1825,7 +1841,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>The `order_date` column in the `purchase_orders` table records the date a purchase order was placed and cannot be null.</t>
+          <t>The `order_date` column in the `purchase_orders` table records the date a purchase order was placed, is mandatory, and uses the `date` data type.</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -1915,7 +1931,11 @@
           <t>The `expected_date` column in the `purchase_orders` table records the anticipated delivery date for a purchase order, allowing null values.</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.OrderDeliveryRelationship</t>
+        </is>
+      </c>
       <c r="L39" t="inlineStr">
         <is>
           <t>temporal.date_only</t>
@@ -1999,7 +2019,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>The `created_at` column records the timestamp when a purchase order record is initially created in the system and cannot be null.</t>
+          <t>The `created_at` column stores the non-nullable timestamp indicating when a purchase order record was initially created in the system.</t>
         </is>
       </c>
       <c r="K40" t="inlineStr"/>
@@ -2086,7 +2106,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>The `updated_at` column stores the non-null timestamp indicating the last modification date and time of a purchase order record.</t>
+          <t>The `updated_at` column stores the non-nullable timestamp of the most recent update to a purchase order record.</t>
         </is>
       </c>
       <c r="K41" t="inlineStr"/>
@@ -2745,7 +2765,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="80" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -2884,7 +2904,11 @@
           <t>Sales line items with sold quantity and explicit unit labels.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.OrderLine, RetailDomainGlossary.SalesOrder, RetailDomainGlossary.UnitOfMeasure</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>{"concept_counts":{"finance.currency_amount":1,"identifier.foreign_key":3,"measure.quantity":3,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":[]}</t>
@@ -3358,10 +3382,14 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Unique identifier for individual items within a sales order, serving as the primary key for the `sales_order_items` table.</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr"/>
+          <t>Unique identifier for each sales order item in the sales_order_items table.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.OrderLine</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -3440,7 +3468,11 @@
           <t>Identifier linking each sales order item to its associated sales order in the `sales_orders` table.</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SalesOrder</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -3520,10 +3552,14 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>References the unique identifier of the product associated with a sales order item, linking to the `products.product_id` column.</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr"/>
+          <t>Identifier for the product associated with the sales order item, referencing the primary key in the products table.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.ProductCategory</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -3607,10 +3643,14 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>The "quantity" column in the "sales_order_items" table stores the non-null integer value representing the number of units of a product included in a specific sales order item.</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
+          <t>The "quantity" column in the "sales_order_items" table stores the number of units of a product included in a sales order item, represented as a non-null integer.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.OrderLine</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>measure.quantity</t>
@@ -3710,10 +3750,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Represents the per-unit price of a product in a sales order item, stored as a non-null numeric value with up to 15 digits and 2 decimal places.</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
+          <t>The `unit_price` column in the `sales_order_items` table stores the per-unit selling price of a product in the sales order as a non-null numeric value with two decimal places.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SellingPrice</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>finance.currency_amount</t>
@@ -3797,7 +3841,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>The `created_at` column in the `sales_order_items` table stores the non-nullable timestamp indicating when a sales order item record was created.</t>
+          <t>Records the timestamp when a sales order item entry is created, ensuring accurate tracking of creation events.</t>
         </is>
       </c>
       <c r="K35" t="inlineStr"/>
@@ -3884,7 +3928,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>The `updated_at` column stores the non-nullable timestamp of the most recent update to a sales order item record for tracking modification history.</t>
+          <t>The `updated_at` column in the `sales_order_items` table stores the non-nullable timestamp of the most recent update to a sales order item record.</t>
         </is>
       </c>
       <c r="K36" t="inlineStr"/>
@@ -3971,10 +4015,14 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Represents the numeric value of the quantity sold for a sales order item, allowing up to two decimal places and nullable for cases where the quantity is not recorded.</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr"/>
+          <t>The `sold_qty_value` column stores the numeric value representing the quantity of a product sold in a sales order item, allowing up to two decimal places, and can be null.</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.OrderLine</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>measure.quantity</t>
@@ -4069,7 +4117,11 @@
           <t>Sold quantity unit (ea/box).</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.UnitOfMeasure</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>measure.quantity</t>
@@ -4648,7 +4700,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="80" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -4787,7 +4839,11 @@
           <t>Sales headers including assigned sales representative relationship.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SalesOrder, RetailDomainGlossary.CustomerIdentifier, RetailDomainGlossary.OrderStatus</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>{"concept_counts":{"entity.status":1,"finance.currency_amount":1,"identifier.foreign_key":5,"temporal.created_at":1,"temporal.date_only":1,"temporal.updated_at":1},"low_confidence_columns":[]}</t>
@@ -5339,10 +5395,14 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Unique identifier for each sales order in the system.</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
+          <t>Unique identifier for each sales order in the system, serving as the primary key for the sales_orders table.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SalesOrder</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -5421,7 +5481,11 @@
           <t>Identifies the store associated with a sales order, referencing the `store_id` column in the `stores` table.</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SalesChannel</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -5505,10 +5569,14 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Identifies the customer associated with a sales order, referencing the `customer_id` column in the `customers` table; nullable to accommodate orders without a registered customer.</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr"/>
+          <t>Represents the identifier of the customer associated with a sales order, referencing the `customer_id` column in the `customers` table, and may be null if no customer is linked.</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.CustomerIdentifier</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -5584,7 +5652,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Identifies the employee responsible for processing the sales order, referencing the `employees.employee_id` column.</t>
+          <t>Represents the unique identifier of the employee associated with the sales order, referencing the `employees.employee_id` column.</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -5761,7 +5829,11 @@
           <t>Indicates the current state of a sales order, such as 'Pending' or 'Completed', stored as a non-nullable text category.</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.OrderStatus</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>entity.status</t>
@@ -5848,7 +5920,11 @@
           <t>The `total_amount` column in the `sales_orders` table stores the non-nullable total monetary value of a sales order as a numeric value with up to 12 digits and 2 decimal places.</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SalesOrder</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>finance.currency_amount</t>
@@ -5932,7 +6008,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>The `created_at` column records the timestamp when a sales order entry was initially created, stored as a non-nullable `datetime2` value.</t>
+          <t>The `created_at` column records the timestamp when a sales order record is initially created, stored as a non-nullable `datetime2` value.</t>
         </is>
       </c>
       <c r="K42" t="inlineStr"/>
@@ -6019,7 +6095,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>The `updated_at` column records the timestamp of the most recent update to a sales order, ensuring accurate tracking of modifications, and it is mandatory.</t>
+          <t>The `updated_at` column records the timestamp of the most recent update to a sales order, stored as a non-nullable datetime2 value.</t>
         </is>
       </c>
       <c r="K43" t="inlineStr"/>
@@ -6814,10 +6890,14 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>The "stores" table contains details about retail store locations, including unique identifiers, names, addresses, contact information, and timestamps for record creation and updates.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>The "stores" table stores information about retail store locations, including unique identifiers, names, codes, addresses, contact details, and timestamps for record creation and updates.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.StoreCode</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>{"concept_counts":{"contact.address":2,"contact.person_name":1,"contact.phone":1,"identifier.foreign_key":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":["address","city","code","name","postal_code","state"]}</t>
@@ -7154,7 +7234,11 @@
           <t>Unique identifier for each store in the retail operations system.</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.StoreCode</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -7230,7 +7314,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>The "name" column in the "stores" table is a non-nullable nvarchar field storing the name of each retail store.</t>
+          <t>The "name" column in the "stores" table is a non-nullable nvarchar field storing the name of a retail store.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -7309,10 +7393,14 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Unique identifier for a store, typically represented as an alphanumeric code.</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr"/>
+          <t>Unique alphanumeric identifier for a store, used for internal reference and operations.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.StoreCode</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
         <v>0.1</v>
@@ -7534,7 +7622,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Indicates the state or province where the store is located, stored as a nullable text field.</t>
+          <t>The "state" column in the "stores" table stores the name of the state or province where a store is located, allowing null values.</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -7609,7 +7697,7 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>The "postal_code" column in the "stores" table stores the postal or ZIP code of a store location as a nullable, case-insensitive string.</t>
+          <t>The "postal_code" column in the "stores" table stores the postal or ZIP code of a store location as a nullable string.</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -7700,7 +7788,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Stores.phone is an optional nvarchar column storing the contact phone number for a store location.</t>
+          <t>The "phone" column in the "stores" table stores the contact phone number of a store as a nullable nvarchar value.</t>
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
@@ -7787,7 +7875,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>The `created_at` column records the non-nullable timestamp indicating when a store record was initially created in the system.</t>
+          <t>The `created_at` column stores the non-nullable timestamp indicating when a store record was initially created in the system.</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -8756,7 +8844,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -8895,7 +8983,11 @@
           <t>The "suppliers" table stores information about suppliers, including their unique identifier, name, contact details, and timestamps for record creation and updates.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SupplierCode</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>{"concept_counts":{"contact.email":1,"contact.person_name":2,"contact.phone":1,"identifier.foreign_key":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":["contact_name","name"]}</t>
@@ -9232,7 +9324,11 @@
           <t>Unique identifier for each supplier, serving as the primary key in the suppliers table.</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SupplierCode</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -9395,7 +9491,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>The `contact_name` column in the `suppliers` table stores the name of the primary contact person for a supplier, allowing null values.</t>
+          <t>Stores the name of the primary contact person for a supplier, allowing null values.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
@@ -9569,7 +9665,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>The "phone" column in the "suppliers" table stores the supplier's contact phone number as a nullable string.</t>
+          <t>The "phone" column in the "suppliers" table stores the contact phone number of a supplier as a nullable string.</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -9656,7 +9752,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>The `created_at` column records the non-nullable timestamp indicating when a supplier record was initially created in the system.</t>
+          <t>Records the timestamp when a supplier entry is initially created in the system, stored as a non-nullable datetime value.</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -9743,7 +9839,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>The `updated_at` column stores the non-nullable timestamp of the most recent update to a supplier record.</t>
+          <t>The `updated_at` column stores the non-nullable timestamp of the most recent update to a supplier record in the `suppliers` table.</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -10326,7 +10422,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"metadata":{"generated_at":"2026-04-03T12:09:52.790221+00:00","database_url":"pioneertest.database.windows.net:1433/free-sql-db-3300567?driver=ODBC+Driver+18+for+SQL+Server&amp;TrustServerCertificate=yes","schema_filter":"dbo","total_tables":10,"total_rows":1364,"total_findings":64},"connection":{"host":"pioneertest.database.windows.net","port":"1433","database":"free-sql-db-3300567","driver":"mssql","timezone":"(UTC) Coordinated Universal Time"},"source_system_context":{"contacts":[],"delete_management_instruction":"","restrictions":"","late_arriving_data_manual":"","volume_size_projection_manual":"","system_description":"Retail operations source system covering customers, stores, employees, suppliers, products, inventory, purchase orders, and sales orders used for day-to-day store, procurement, and sales transaction management.","openmetadata_enrichment":{"enabled":false,"configured":false,"database_service_name":"","schema":"dbo","matched_tables":0,"unmatched_tables":0,"error":""},"db_analysis_config":{"exclude_schemas":["prediction"],"exclude_tables":[],"max_row_limit":100}},"concept_registry":{"version":1,"taxonomy":"domain-dot","generated_from_tables":10,"concepts":[{"concept_id":"contact.address","column_count":2,"table_count":1,"avg_confidence":0.55,"alias_groups":["address","postal_code"],"sample_columns":["stores.address","stores.postal_code"],"signals":["name","type"]},{"concept_id":"contact.email","column_count":3,"table_count":3,"avg_confidence":1.0,"alias_groups":["email"],"sample_columns":["customers.email","employees.email","suppliers.email"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"contact.person_name","column_count":8,"table_count":5,"avg_confidence":0.56,"alias_groups":["contact_name","first_name","last_name","name"],"sample_columns":["customers.first_name","customers.last_name","employees.first_name","employees.last_name","products.name"],"signals":["name","table_context","type"]},{"concept_id":"contact.phone","column_count":3,"table_count":3,"avg_confidence":1.0,"alias_groups":["phone"],"sample_columns":["customers.phone","stores.phone","suppliers.phone"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"entity.category","column_count":1,"table_count":1,"avg_confidence":0.8,"alias_groups":["category"],"sample_columns":["products.category"],"signals":["name","profile","type"]},{"concept_id":"entity.status","column_count":2,"table_count":2,"avg_confidence":1.0,"alias_groups":["statu"],"sample_columns":["purchase_orders.status","sales_orders.status"],"signals":["name","profile","type","values"]},{"concept_id":"entity.type","column_count":1,"table_count":1,"avg_confidence":0.65,"alias_groups":["role"],"sample_columns":["employees.role"],"signals":["name","profile","type"]},{"concept_id":"finance.currency_amount","column_count":5,"table_count":4,"avg_confidence":1.0,"alias_groups":["amount","price","unit_cost"],"sample_columns":["products.unit_price","products.cost_price","purchase_order_items.unit_cost","sales_order_items.unit_price","sales_orders.total_amount"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"identifier.foreign_key","column_count":26,"table_count":10,"avg_confidence":0.78,"alias_groups":["id"],"sample_columns":["customers.customer_id","employees.employee_id","employees.store_id","inventory.inventory_id","inventory.store_id"],"signals":["cross_table_consensus","name","profile","type"]},{"concept_id":"identifier.product_code","column_count":1,"table_count":1,"avg_confidence":0.7,"alias_groups":["sku"],"sample_columns":["products.sku"],"signals":["name","profile","type"]},{"concept_id":"measure.quantity","column_count":7,"table_count":3,"avg_confidence":1.0,"alias_groups":["ordered_qty","ordered_qty_unit","quantity","quantity_on_hand","sold_qty","sold_qty_unit"],"sample_columns":["inventory.quantity_on_hand","purchase_order_items.quantity","purchase_order_items.ordered_qty_value","purchase_order_items.ordered_qty_unit","sales_order_items.quantity"],"signals":["name","profile","type","values"]},{"concept_id":"temporal.created_at","column_count":10,"table_count":10,"avg_confidence":1.0,"alias_groups":["created_at"],"sample_columns":["customers.created_at","employees.created_at","inventory.created_at","products.created_at","purchase_order_items.created_at"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"temporal.date_only","column_count":4,"table_count":3,"avg_confidence":0.97,"alias_groups":["expected_date","hire_date","order_date"],"sample_columns":["employees.hire_date","purchase_orders.order_date","purchase_orders.expected_date","sales_orders.order_date"],"signals":["cross_table_consensus","name","profile","table_context","type","values"]},{"concept_id":"temporal.event_time","column_count":1,"table_count":1,"avg_confidence":1.0,"alias_groups":["last_restocked_at"],"sample_columns":["inventory.last_restocked_at"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"temporal.updated_at","column_count":10,"table_count":10,"avg_confidence":1.0,"alias_groups":["updated_at"],"sample_columns":["customers.updated_at","employees.updated_at","inventory.updated_at","products.updated_at","purchase_order_items.updated_at"],"signals":["name","profile","table_context","type","values"]}]},"data_quality_summary":{"critical":0,"warning":27,"info":37,"by_check":{"controlled_value_candidate":7,"nullable_but_never_null":13,"missing_primary_key":0,"missing_foreign_key":0,"format_inconsistency":0,"range_violation":0,"timestamp_ordering":10,"delete_management":10,"late_arriving_data":3,"timezone":10,"unit_unknown":11,"unit_noncanonical_but_convertible":0,"unit_mismatch_within_semantic_group":0},"constraints_found":{"check_constraints":0,"enum_columns":0,"unique_constraints":10}},"tables":[{"table":"customers","schema":"dbo","columns":[{"name":"customer_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each customer in the retail operations system.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"404","max":"503"},"data_category":"discrete","semantic_class":"customer_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"first_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Stores the given name of a customer as a non-null, case-insensitive Unicode string.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"Customer1","max":"Customer99"},"data_category":"nominal","semantic_class":"given_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.6,"concept_evidence":["name token: first_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","table context: customers"],"concept_sources":["name","table_context","type"],"concept_alias_group":"first_name"},{"name":"last_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Stores the last name of a customer as a non-null, case-insensitive Unicode string.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"LastName1 (updated)","max":"LastName99"},"data_category":"nominal","semantic_class":"family_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.6,"concept_evidence":["name token: last_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","table context: customers"],"concept_sources":["name","table_context","type"],"concept_alias_group":"last_name"},{"name":"email","type":"nvarchar(450)","nullable":true,"is_incremental":false,"column_description":"Stores the email address of the customer, allowing null values.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"customer1@example.com","max":"customer99@example.com"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.email","concept_confidence":1.0,"concept_evidence":["name token: email","type hint: nvarchar(450)","legacy field classification: contact","value pattern: email","table context: customers","sensitive hint: pii_contact"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"email"},{"name":"phone","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"Stores the customer's phone number as an optional text field for contact purposes.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"555-1001","max":"555-1100"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.phone","concept_confidence":1.0,"concept_evidence":["name token: phone","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: contact","value pattern: phone","table context: customers","sensitive hint: pii_contact"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"phone"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the non-nullable timestamp indicating when a customer record was initially created in the system.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":95,"null_count":0,"data_range":{"min":"2021-03-23 15:38:57.201565","max":"2026-02-26 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: customers"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"Tracks the timestamp of the most recent update to a customer's record, ensuring accurate change history.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":95,"null_count":0,"data_range":{"min":"2021-03-23 15:38:57.201565","max":"2026-03-26 08:52:49.252228"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: customers"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"}],"table_description":"The `customers` table stores information about retail customers, including their unique ID, name, contact details, and timestamps for record creation and updates.","glossary_terms":[],"primary_keys":["customer_id"],"foreign_keys":[],"row_count":100,"field_classifications":{"customer_id":"identifier","first_name":"person_name","last_name":"person_name","email":"contact","phone":"contact","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{"email":"pii_contact","phone":"pii_contact"},"incremental_columns":["updated_at"],"join_candidates":[],"unit_summary":{"columns_with_units":0,"columns_without_units":7,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":false,"has_sensitive_fields":true,"row_count_projection_1y":126,"row_count_projection_2y":152,"row_count_projection_5y":232,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.email":1,"contact.person_name":2,"contact.phone":1,"identifier.foreign_key":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":"email","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 100 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"phone","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 100 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}},{"table":"employees","schema":"dbo","columns":[{"name":"employee_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each employee in the retail operations system.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"64","max":"83"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Associates each employee with a specific store, referencing the `store_id` column in the `stores` table.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"first_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Stores the given name of an employee, represented as a non-null, case-insensitive Unicode string.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"Employee1","max":"Employee9"},"data_category":"nominal","semantic_class":"given_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: first_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"first_name"},{"name":"last_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"The \"last_name\" column in the \"employees\" table stores the non-nullable family name of an employee as a case-insensitive Unicode string.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"LastName1","max":"LastName9"},"data_category":"nominal","semantic_class":"family_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: last_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"last_name"},{"name":"email","type":"nvarchar(450)","nullable":false,"is_incremental":false,"column_description":"Stores the unique email address of each employee for contact purposes, with a maximum length of 450 characters and cannot be null.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"emp1@example.com","max":"emp9@example.com"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.email","concept_confidence":1.0,"concept_evidence":["name token: email","type hint: nvarchar(450)","legacy field classification: contact","value pattern: email","sensitive hint: pii_contact"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"email"},{"name":"role","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Indicates the job position or function of an employee within the organization, stored as a non-nullable text value.","glossary_terms":[],"cardinality":4,"null_count":0,"data_range":{"min":"Cashier","max":"Stock"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"entity.type","concept_confidence":0.65,"concept_evidence":["name token: role","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","profile heuristic matched"],"concept_sources":["name","profile","type"],"concept_alias_group":"role"},{"name":"hire_date","type":"date","nullable":false,"is_incremental":false,"column_description":"The `hire_date` column in the `employees` table stores the non-nullable date an employee was hired, used for tracking employment start dates.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"2021-05-03","max":"2025-01-26"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.date_only","concept_confidence":1.0,"concept_evidence":["name token: hire_date","type hint: date","legacy field classification: temporal","value pattern: date_only","table context: employees"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"hire_date"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the non-nullable timestamp indicating when an employee record was initially created in the system.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":20,"null_count":0,"data_range":{"min":"2021-05-03 15:38:57.201565","max":"2025-01-26 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: employees"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column stores the non-nullable timestamp of the most recent update to an employee record.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":20,"null_count":0,"data_range":{"min":"2021-05-03 15:38:57.201565","max":"2025-01-26 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: employees"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"}],"table_description":"The `employees` table stores details about retail system employees, including their identifiers, store associations, personal information, roles, hire dates, and record timestamps.","glossary_terms":[],"primary_keys":["employee_id"],"foreign_keys":[{"column":"store_id","references":"stores.store_id"}],"row_count":20,"field_classifications":{"first_name":"person_name","last_name":"person_name","email":"contact","hire_date":"temporal","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{"email":"pii_contact"},"incremental_columns":["updated_at"],"join_candidates":[{"column":"store_id","target_table":"stores","target_column":"store_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":9,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":true,"row_count_projection_1y":35,"row_count_projection_2y":50,"row_count_projection_5y":96,"partition_columns_candidates":["hire_date","created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.email":1,"contact.person_name":2,"entity.type":1,"identifier.foreign_key":2,"temporal.created_at":1,"temporal.date_only":1,"temporal.updated_at":1},"low_confidence_columns":["first_name","last_name"]},"data_quality":{"findings":[{"column":"role","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 4 distinct value(s) ('Cashier', 'Manager', 'Sales', 'Stock') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Cashier","Manager","Sales","Stock"],"cardinality":4},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":"hire_date","check":"late_arriving_data","severity":"info","detail":"Minor arrival delay \u2014 max lag between 'hire_date' and 'created_at' is 15.7h (avg 15.7h, P95 15.7h).","recommendation":"Use 'created_at' as the watermark (preferred). If using 'hire_date', add a 1\u20132 day lookback buffer.","business_date_column":"hire_date","system_ts_column":"created_at","lag_stats":{"total_rows_compared":20,"min_lag_hours":15.65,"avg_lag_hours":15.65,"p95_lag_hours":15.65,"max_lag_hours":15.65,"max_lag_days":0.7,"rows_late_over_1d":0,"rows_late_over_7d":0},"recommended_lookback_days":2},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}},{"table":"inventory","schema":"dbo","columns":[{"name":"inventory_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each inventory record in the system.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"8","max":"107"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifier for the store associated with the inventory record, referencing the `store_id` column in the `stores` table.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"product_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"References the unique identifier of a product from the `products` table to associate inventory records with specific products.","glossary_terms":[],"cardinality":47,"null_count":0,"data_range":{"min":"156","max":"205"},"data_category":"discrete","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"quantity_on_hand","type":"integer","nullable":false,"is_incremental":false,"column_description":"Tracks the current quantity of a product available in inventory, expressed as a non-null integer.","glossary_terms":[],"cardinality":68,"null_count":0,"data_range":{"min":"2","max":"98"},"data_category":"discrete","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: quantity_on_hand","type hint: integer","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"quantity_on_hand"},{"name":"reorder_level","type":"integer","nullable":false,"is_incremental":false,"column_description":"Indicates the minimum quantity of a product in inventory that triggers a reorder, stored as a non-null integer.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"10","max":"29"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: integer","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"last_restocked_at","type":"datetime2","nullable":true,"is_incremental":false,"column_description":"The `last_restocked_at` column records the timestamp of the most recent restocking event for an inventory item, allowing null values if the item has not been restocked.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":89,"null_count":0,"data_range":{"min":"2024-03-14 15:38:57.201565","max":"2026-03-07 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.event_time","concept_confidence":1.0,"concept_evidence":["name token: last_restocked_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: inventory"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"last_restocked_at"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the non-nullable timestamp indicating when the inventory record was initially created.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":91,"null_count":0,"data_range":{"min":"2024-03-05 15:38:57.201565","max":"2026-02-23 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: inventory"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"Tracks the timestamp of the most recent update to an inventory record, ensuring accurate change history.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":89,"null_count":0,"data_range":{"min":"2024-03-14 15:38:57.201565","max":"2026-03-07 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"conc</t>
+          <t>{"metadata":{"generated_at":"2026-04-07T08:55:59.245988+00:00","database_url":"pioneertest.database.windows.net:1433/free-sql-db-3300567?driver=ODBC+Driver+18+for+SQL+Server&amp;TrustServerCertificate=yes","schema_filter":"dbo","total_tables":10,"total_rows":1364,"total_findings":64},"connection":{"host":"pioneertest.database.windows.net","port":"1433","database":"free-sql-db-3300567","driver":"mssql","timezone":"(UTC) Coordinated Universal Time"},"source_system_context":{"contacts":[],"delete_management_instruction":"","restrictions":"","late_arriving_data_manual":"","volume_size_projection_manual":"","system_description":"Retail operations source system covering customers, stores, employees, suppliers, products, inventory, purchase orders, and sales orders used for day-to-day store, procurement, and sales transaction management.","openmetadata_enrichment":{"enabled":true,"configured":true,"database_service_name":"","schema":"dbo","match_strategy":"table_name","matched_tables":0,"unmatched_tables":10,"error":""},"db_analysis_config":{"exclude_schemas":["prediction"],"exclude_tables":[],"max_row_limit":100}},"concept_registry":{"version":1,"taxonomy":"domain-dot","generated_from_tables":10,"concepts":[{"concept_id":"contact.address","column_count":2,"table_count":1,"avg_confidence":0.55,"alias_groups":["address","postal_code"],"sample_columns":["stores.address","stores.postal_code"],"signals":["name","type"]},{"concept_id":"contact.email","column_count":3,"table_count":3,"avg_confidence":1.0,"alias_groups":["email"],"sample_columns":["customers.email","employees.email","suppliers.email"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"contact.person_name","column_count":8,"table_count":5,"avg_confidence":0.56,"alias_groups":["contact_name","first_name","last_name","name"],"sample_columns":["customers.first_name","customers.last_name","employees.first_name","employees.last_name","products.name"],"signals":["name","table_context","type"]},{"concept_id":"contact.phone","column_count":3,"table_count":3,"avg_confidence":1.0,"alias_groups":["phone"],"sample_columns":["customers.phone","stores.phone","suppliers.phone"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"entity.category","column_count":1,"table_count":1,"avg_confidence":0.8,"alias_groups":["category"],"sample_columns":["products.category"],"signals":["name","profile","type"]},{"concept_id":"entity.status","column_count":2,"table_count":2,"avg_confidence":1.0,"alias_groups":["statu"],"sample_columns":["purchase_orders.status","sales_orders.status"],"signals":["name","profile","type","values"]},{"concept_id":"entity.type","column_count":1,"table_count":1,"avg_confidence":0.65,"alias_groups":["role"],"sample_columns":["employees.role"],"signals":["name","profile","type"]},{"concept_id":"finance.currency_amount","column_count":5,"table_count":4,"avg_confidence":1.0,"alias_groups":["amount","price","unit_cost"],"sample_columns":["products.unit_price","products.cost_price","purchase_order_items.unit_cost","sales_order_items.unit_price","sales_orders.total_amount"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"identifier.foreign_key","column_count":26,"table_count":10,"avg_confidence":0.78,"alias_groups":["id"],"sample_columns":["customers.customer_id","employees.employee_id","employees.store_id","inventory.inventory_id","inventory.store_id"],"signals":["cross_table_consensus","name","profile","type"]},{"concept_id":"identifier.product_code","column_count":1,"table_count":1,"avg_confidence":0.7,"alias_groups":["sku"],"sample_columns":["products.sku"],"signals":["name","profile","type"]},{"concept_id":"measure.quantity","column_count":7,"table_count":3,"avg_confidence":1.0,"alias_groups":["ordered_qty","ordered_qty_unit","quantity","quantity_on_hand","sold_qty","sold_qty_unit"],"sample_columns":["inventory.quantity_on_hand","purchase_order_items.quantity","purchase_order_items.ordered_qty_value","purchase_order_items.ordered_qty_unit","sales_order_items.quantity"],"signals":["name","profile","type","values"]},{"concept_id":"temporal.created_at","column_count":10,"table_count":10,"avg_confidence":1.0,"alias_groups":["created_at"],"sample_columns":["customers.created_at","employees.created_at","inventory.created_at","products.created_at","purchase_order_items.created_at"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"temporal.date_only","column_count":4,"table_count":3,"avg_confidence":0.97,"alias_groups":["expected_date","hire_date","order_date"],"sample_columns":["employees.hire_date","purchase_orders.order_date","purchase_orders.expected_date","sales_orders.order_date"],"signals":["cross_table_consensus","name","profile","table_context","type","values"]},{"concept_id":"temporal.event_time","column_count":1,"table_count":1,"avg_confidence":1.0,"alias_groups":["last_restocked_at"],"sample_columns":["inventory.last_restocked_at"],"signals":["name","profile","table_context","type","values"]},{"concept_id":"temporal.updated_at","column_count":10,"table_count":10,"avg_confidence":1.0,"alias_groups":["updated_at"],"sample_columns":["customers.updated_at","employees.updated_at","inventory.updated_at","products.updated_at","purchase_order_items.updated_at"],"signals":["name","profile","table_context","type","values"]}]},"data_quality_summary":{"critical":0,"warning":27,"info":37,"by_check":{"controlled_value_candidate":7,"nullable_but_never_null":13,"missing_primary_key":0,"missing_foreign_key":0,"format_inconsistency":0,"range_violation":0,"timestamp_ordering":10,"delete_management":10,"late_arriving_data":3,"timezone":10,"unit_unknown":11,"unit_noncanonical_but_convertible":0,"unit_mismatch_within_semantic_group":0},"constraints_found":{"check_constraints":0,"enum_columns":0,"unique_constraints":10}},"tables":[{"table":"customers","schema":"dbo","columns":[{"name":"customer_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each customer in the retail operations system.","glossary_terms":["RetailDomainGlossary.CustomerIdentifier"],"cardinality":100,"null_count":0,"data_range":{"min":"404","max":"503"},"data_category":"discrete","semantic_class":"customer_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"first_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Stores the given name of a customer as a non-null Unicode string.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"Customer1","max":"Customer99"},"data_category":"nominal","semantic_class":"given_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.6,"concept_evidence":["name token: first_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","table context: customers"],"concept_sources":["name","table_context","type"],"concept_alias_group":"first_name"},{"name":"last_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"The \"last_name\" column in the \"customers\" table stores the non-nullable family name of a customer as a case-insensitive Unicode string.","glossary_terms":["RetailDomainGlossary.Customer"],"cardinality":100,"null_count":0,"data_range":{"min":"LastName1 (updated)","max":"LastName99"},"data_category":"nominal","semantic_class":"family_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.6,"concept_evidence":["name token: last_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","table context: customers"],"concept_sources":["name","table_context","type"],"concept_alias_group":"last_name"},{"name":"email","type":"nvarchar(450)","nullable":true,"is_incremental":false,"column_description":"Stores the email address of the customer, allowing null values for cases where an email is not provided.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"customer1@example.com","max":"customer99@example.com"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.email","concept_confidence":1.0,"concept_evidence":["name token: email","type hint: nvarchar(450)","legacy field classification: contact","value pattern: email","table context: customers","sensitive hint: pii_contact"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"email"},{"name":"phone","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"Stores the customer's phone number as an optional text field for contact purposes.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"555-1001","max":"555-1100"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.phone","concept_confidence":1.0,"concept_evidence":["name token: phone","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: contact","value pattern: phone","table context: customers","sensitive hint: pii_contact"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"phone"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the non-nullable timestamp indicating when a customer record was initially created in the system.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":95,"null_count":0,"data_range":{"min":"2021-03-23 15:38:57.201565","max":"2026-02-26 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: customers"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"Tracks the timestamp of the most recent update to a customer record, ensuring accurate audit and change history.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":95,"null_count":0,"data_range":{"min":"2021-03-23 15:38:57.201565","max":"2026-03-26 08:52:49.252228"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: customers"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"}],"table_description":"The \"customers\" table stores information about retail customers, including their unique ID, name, contact details, and timestamps for record creation and updates.","glossary_terms":["RetailDomainGlossary.CustomerIdentifier"],"primary_keys":["customer_id"],"foreign_keys":[],"row_count":100,"field_classifications":{"customer_id":"identifier","first_name":"person_name","last_name":"person_name","email":"contact","phone":"contact","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{"email":"pii_contact","phone":"pii_contact"},"incremental_columns":["updated_at"],"join_candidates":[],"unit_summary":{"columns_with_units":0,"columns_without_units":7,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":false,"has_sensitive_fields":true,"row_count_projection_1y":126,"row_count_projection_2y":152,"row_count_projection_5y":232,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.email":1,"contact.person_name":2,"contact.phone":1,"identifier.foreign_key":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":"email","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 100 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"phone","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 100 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}},{"table":"employees","schema":"dbo","columns":[{"name":"employee_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for employees in the retail operations system.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"64","max":"83"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifies the store where the employee is assigned, referencing the `store_id` column in the `stores` table.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"first_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Stores the given name of an employee, represented as a non-null Unicode string.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"Employee1","max":"Employee9"},"data_category":"nominal","semantic_class":"given_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: first_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"first_name"},{"name":"last_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"The \"last_name\" column in the \"employees\" table stores the non-nullable family name of each employee as a case-insensitive Unicode string.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"LastName1","max":"LastName9"},"data_category":"nominal","semantic_class":"family_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: last_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"last_name"},{"name":"email","type":"nvarchar(450)","nullable":false,"is_incremental":false,"column_description":"The \"email\" column in the \"employees\" table stores the unique, non-null email address of each employee for contact purposes.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"emp1@example.com","max":"emp9@example.com"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.email","concept_confidence":1.0,"concept_evidence":["name token: email","type hint: nvarchar(450)","legacy field classification: contact","value pattern: email","sensitive hint: pii_contact"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"email"},{"name":"role","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Stores the job role or position of an employee within the organization, such as \"Cashier\" or \"Sales,\" as a non-null text value.","glossary_terms":[],"cardinality":4,"null_count":0,"data_range":{"min":"Cashier","max":"Stock"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"entity.type","concept_confidence":0.65,"concept_evidence":["name token: role","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","profile heuristic matched"],"concept_sources":["name","profile","type"],"concept_alias_group":"role"},{"name":"hire_date","type":"date","nullable":false,"is_incremental":false,"column_description":"The `hire_date` column in the `employees` table stores the non-nullable date an employee was hired, used for tracking employment start dates.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"2021-05-03","max":"2025-01-26"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.date_only","concept_confidence":1.0,"concept_evidence":["name token: hire_date","type hint: date","legacy field classification: temporal","value pattern: date_only","table context: employees"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"hire_date"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the non-nullable timestamp indicating when an employee record was initially created in the system.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":20,"null_count":0,"data_range":{"min":"2021-05-03 15:38:57.201565","max":"2025-01-26 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: employees"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column in the `employees` table stores the non-nullable timestamp of the most recent update to an employee record.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":20,"null_count":0,"data_range":{"min":"2021-05-03 15:38:57.201565","max":"2025-01-26 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: employees"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"}],"table_description":"The `employees` table stores detailed information about retail system employees, including their unique identifiers, store assignments, personal details, job roles, hire dates, and record timestamps.","glossary_terms":[],"primary_keys":["employee_id"],"foreign_keys":[{"column":"store_id","references":"stores.store_id"}],"row_count":20,"field_classifications":{"first_name":"person_name","last_name":"person_name","email":"contact","hire_date":"temporal","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{"email":"pii_contact"},"incremental_columns":["updated_at"],"join_candidates":[{"column":"store_id","target_table":"stores","target_column":"store_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":9,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":true,"row_count_projection_1y":35,"row_count_projection_2y":50,"row_count_projection_5y":96,"partition_columns_candidates":["hire_date","created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.email":1,"contact.person_name":2,"entity.type":1,"identifier.foreign_key":2,"temporal.created_at":1,"temporal.date_only":1,"temporal.updated_at":1},"low_confidence_columns":["first_name","last_name"]},"data_quality":{"findings":[{"column":"role","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 4 distinct value(s) ('Cashier', 'Manager', 'Sales', 'Stock') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Cashier","Manager","Sales","Stock"],"cardinality":4},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":"hire_date","check":"late_arriving_data","severity":"info","detail":"Minor arrival delay \u2014 max lag between 'hire_date' and 'created_at' is 15.7h (avg 15.7h, P95 15.7h).","recommendation":"Use 'created_at' as the watermark (preferred). If using 'hire_date', add a 1\u20132 day lookback buffer.","business_date_column":"hire_date","system_ts_column":"created_at","lag_stats":{"total_rows_compared":20,"min_lag_hours":15.65,"avg_lag_hours":15.65,"p95_lag_hours":15.65,"max_lag_hours":15.65,"max_lag_days":0.7,"rows_late_over_1d":0,"rows_late_over_7d":0},"recommended_lookback_days":2},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}},{"table":"inventory","schema":"dbo","columns":[{"name":"inventory_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each inventory record in the system.","glossary_terms":[],"cardinality":100,"null_count":0,"data_range":{"min":"8","max":"107"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Represents the unique identifier of the store associated with the inventory record, referencing the `store_id` column in the `stores` table.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"product_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"References the unique identifier of a product from the products table, linking inventory records to specific products.","glossary_terms":[],"cardinality":47,"null_count":0,"data_range":{"min":"156","max":"205"},"data_category":"discrete","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"quantity_on_hand","type":"integer","nullable":false,"is_incremental":false,"column_description":"The `quantity_on_hand` column in the `inventory` table stores the current stock level of a product as a non-null integer.","glossary_terms":["RetailDomainGlossary.Inventory"],"cardinality":68,"null_count":0,"data_range":{"min":"2","max":"98"},"data_category":"discrete","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: quantity_on_hand","type hint: integer","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"quantity_on_hand"},{"name":"reorder_level","type":"integer","nullable":false,"is_incremental":false,"column_description":"Indicates the minimum quantity of a product in inventory that triggers a reorder, stored as a non-null integer.","glossary_terms":["RetailDomainGlossary.ReorderPoint"],"cardinality":20,"null_count":0,"data_range":{"min":"10","max":"29"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: integer","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"last_restocked_at","type":"datetime2","nullable":true,"is_incremental":false,"column_description":"The `last_restocked_at` column records the timestamp of the most recent restocking event for an inventory item, allowing null values if the item has not been restocked.","glossary_terms":["RetailDomainGlossary.Replenishment"],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":89,"null_count":0,"data_range":{"min":"2024-03-14 15:38:57.201565","max":"2026-03-07 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.event_time","concept_confidence":1.0,"concept_evidence":["name token: last_restocked_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: inventory"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"last_restocked_at"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the non-nullable timestamp indicating when the inventory record was initially created.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":91,"null_count":0,"data_range":{"min":"2024-03-05 15:38:57.201565","max":"2026-02-23 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: inventory"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incr</t>
         </is>
       </c>
     </row>
@@ -10336,7 +10432,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: inventory"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"stock_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"Represents the monetary value of inventory stock, stored as a numeric value with up to 10 digits and 2 decimal places, and may be null.","glossary_terms":[],"cardinality":0,"null_count":100,"data_category":"continuous","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.0,"concept_evidence":["type hint: numeric(10,2)","ambiguous runner-up concept"],"concept_sources":["type"],"concept_alias_group":null},{"name":"stock_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Current stock unit label.","glossary_terms":[],"cardinality":0,"null_count":100,"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.15,"concept_evidence":["value pattern: quantity","ambiguous runner-up concept"],"concept_sources":["values"],"concept_alias_group":null}],"table_description":"Current stock levels with normalized stock unit representation.","glossary_terms":[],"primary_keys":["inventory_id"],"foreign_keys":[{"column":"product_id","references":"products.product_id"},{"column":"store_id","references":"stores.store_id"}],"row_count":100,"field_classifications":{"quantity_on_hand":"quantity","last_restocked_at":"temporal","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"product_id","target_table":"products","target_column":"product_id","confidence":"high"},{"column":"store_id","target_table":"stores","target_column":"store_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":10,"mixed_unit_groups":[],"unknown_unit_columns":["quantity_on_hand"]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":146,"row_count_projection_2y":193,"row_count_projection_5y":334,"partition_columns_candidates":["last_restocked_at","created_at","updated_at"],"classification_summary":{"concept_counts":{"identifier.foreign_key":3,"measure.quantity":1,"temporal.created_at":1,"temporal.event_time":1,"temporal.updated_at":1},"low_confidence_columns":["reorder_level","stock_unit"]},"data_quality":{"findings":[{"column":"last_restocked_at","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 100 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 3 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"last_restocked_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":3},{"column":"quantity_on_hand","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."}]}},{"table":"products","schema":"dbo","columns":[{"name":"product_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each product in the retail operations system.","glossary_terms":[],"cardinality":50,"null_count":0,"data_range":{"min":"156","max":"205"},"data_category":"discrete","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"supplier_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"The `supplier_id` column in the `products` table is a non-nullable foreign key referencing the `supplier_id` column in the `suppliers` table, identifying the supplier associated with each product.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"33","max":"42"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"sku","type":"nvarchar(450)","nullable":false,"is_incremental":false,"column_description":"Unique alphanumeric identifier for a product used for inventory and sales tracking, stored as a non-null nvarchar(450).","glossary_terms":[],"cardinality":50,"null_count":0,"data_range":{"min":"SKU-0001","max":"SKU-0050"},"data_category":"nominal","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.product_code","concept_confidence":0.7,"concept_evidence":["name token: sku","type hint: nvarchar(450)","semantic class hint: product_identifier"],"concept_sources":["name","profile","type"],"concept_alias_group":"sku"},{"name":"name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"The \"name\" column in the \"products\" table stores the non-nullable name of a product as a case-insensitive Unicode string.","glossary_terms":[],"cardinality":50,"null_count":0,"data_range":{"min":"Product 1","max":"Product 9"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"name"},{"name":"category","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Indicates the product's category classification, such as \"Books,\" \"Clothing,\" or \"Electronics,\" stored as a non-null, case-insensitive text value.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"Books","max":"Sports"},"data_category":"nominal","semantic_class":"category","unit_context":null,"concept_id":"entity.category","concept_confidence":0.8,"concept_evidence":["name token: category","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: categorical","profile heuristic matched"],"concept_sources":["name","profile","type"],"concept_alias_group":"category"},{"name":"unit_price","type":"numeric(10,2)","nullable":false,"is_incremental":false,"column_description":"Stores the retail price of a product as a non-null numeric value with up to 10 digits and 2 decimal places.","glossary_terms":[],"cardinality":50,"null_count":0,"data_range":{"min":"11.09","max":"490.43"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: price","type hint: numeric(10,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"price"},{"name":"cost_price","type":"numeric(10,2)","nullable":false,"is_incremental":false,"column_description":"Represents the numeric cost price of a product in the retail system, stored as a non-nullable currency amount with up to 10 digits and 2 decimal places.","glossary_terms":[],"cardinality":50,"null_count":0,"data_range":{"min":"5.55","max":"358.59"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: price","type hint: numeric(10,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"price"},{"name":"active","type":"bit","nullable":false,"is_incremental":false,"column_description":"Indicates whether a product is active and available for transactions, stored as a non-nullable boolean value.","glossary_terms":[],"cardinality":1,"null_count":0,"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.0,"concept_evidence":["profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile"],"concept_alias_group":null},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"Indicates the timestamp when the product record was initially created, stored as a non-nullable datetime value.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":50,"null_count":0,"data_range":{"min":"2021-03-20 15:38:57.201565","max":"2024-12-25 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: products"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column stores the non-nullable timestamp of the most recent update to a product record in the `products` table.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":50,"null_count":0,"data_range":{"min":"2021-03-20 15:38:57.201565","max":"2024-12-25 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: products"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"weight_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Source weight unit (kg/lb) used for unit inference testing.","glossary_terms":[],"cardinality":0,"null_count":50,"data_category":"nominal","semantic_class":"mass","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":null,"concept_confidence":0.15,"concept_evidence":["value pattern: quantity","ambiguous runner-up concept"],"concept_sources":["values"],"concept_alias_group":null},{"name":"weight_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"The `weight_value` column stores the weight of a product as a numeric value with up to 10 digits and 2 decimal places, and it is nullable.","glossary_terms":[],"cardinality":0,"null_count":50,"data_category":"continuous","semantic_class":"mass","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":null,"concept_confidence":0.0,"concept_evidence":["type hint: numeric(10,2)","ambiguous runner-up concept"],"concept_sources":["type"],"concept_alias_group":null},{"name":"length_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"The \"length_value\" column stores the numeric length measurement of a product, allowing up to 10 digits with 2 decimal places, and is nullable.","glossary_terms":[],"cardinality":0,"null_count":50,"data_category":"continuous","semantic_class":"length","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":null,"concept_confidence":0.0,"concept_evidence":["type hint: numeric(10,2)","ambiguous runner-up concept"],"concept_sources":["type"],"concept_alias_group":null},{"name":"length_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Source length unit (cm/in) used for unit inference testing.","glossary_terms":[],"cardinality":0,"null_count":50,"data_category":"nominal","semantic_class":"length","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":null,"concept_confidence":0.15,"concept_evidence":["value pattern: quantity","ambiguous runner-up concept"],"concept_sources":["values"],"concept_alias_group":null},{"name":"product_description","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"Stores optional textual details about a product, such as features or specifications, with support for Unicode characters.","glossary_terms":[],"cardinality":0,"null_count":50,"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"primary_supplier_id","type":"bigint","nullable":true,"is_incremental":false,"column_description":"Primary supplier relationship used for join candidate detection.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"33","max":"42"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"}],"table_description":"Master product catalog including physical units for analyzer unit-context testing.","glossary_terms":[],"primary_keys":["product_id"],"foreign_keys":[{"column":"primary_supplier_id","references":"suppliers.supplier_id"},{"column":"supplier_id","references":"suppliers.supplier_id"}],"row_count":50,"field_classifications":{"category":"categorical","unit_price":"pricing","cost_price":"pricing","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"primary_supplier_id","target_table":"suppliers","target_column":"supplier_id","confidence":"high"},{"column":"supplier_id","target_table":"suppliers","target_column":"supplier_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":16,"mixed_unit_groups":[],"unknown_unit_columns":["length_unit","length_value","weight_unit","weight_value"]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":68,"row_count_projection_2y":86,"row_count_projection_5y":141,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.person_name":1,"entity.category":1,"finance.currency_amount":2,"identifier.foreign_key":3,"identifier.product_code":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":["length_unit","name","product_description","weight_unit"]},"data_quality":{"findings":[{"column":"category","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 5 distinct value(s) ('Books', 'Clothing', 'Electronics', 'Home', 'Sports') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Books","Clothing","Electronics","Home","Sports"],"cardinality":5},{"column":"primary_supplier_id","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 50 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":"active","check":"delete_management","severity":"info","detail":"Active-flag column 'active' (boolean) detected \u2014 rows with active=false are logically deleted. Current distribution: True=50.","recommendation":"Filter on \"active\" = true for current records during ingestion.","delete_strategy":"soft_delete","soft_delete_column":"active","soft_delete_type":"active_flag","has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2},{"column":"weight_unit","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'mass' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"weight_value","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'mass' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"length_value","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'length' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"length_unit","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'length' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."}]}},{"table":"purchase_order_items","schema":"dbo","columns":[{"name":"po_item_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each purchase order item record in the `purchase_order_items` table.","glossary_terms":[],"cardinality":246,"null_count":0,"data_range":{"min":"268","max":"513"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"po_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Links each purchase order item to its corresponding purchase order in the `purchase_orders` table via a non-null foreign key.","glossary_terms":[],"cardinality":125,"null_count":0,"data_range":{"min":"128","max":"252"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"product_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifier linking each purchase order item to a specific product in the products table.","glossary_terms":[],"cardinality":49,"null_count":0,"data_range":{"min":"156","max":"205"},"data_category":"discrete","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"quantity","type":"integer","nullable":false,"is_incremental":false,"column_description":"The `quantity` column in the `purchase_order_items` table stores the non-null integer value representing the number of units of a product included in a specific purchase order item.","glossary_terms":[],"cardinality":41,"null_count":0,"data_range":{"min":"10","max":"50"},"data_category":"discrete","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: quantity","type hint: integer","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"quantity"},{"name":"unit_cost","type":"numeric(10,2)","nullable":false,"is_incremental":false,"column_description":"The `unit_cost` column in the `purchase_order_items` table stores the non-null numeric cost per unit of a product in a purchase order, represented as a currency amount with up to 10 digits and 2 decimal places.","glossary_terms":[],"cardinality":49,"null_count":0,"data_range":{"min":"5.55","max":"358.59"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: unit_cost","type hint: numeric(10,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount","table context: purchase_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"unit_cost"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"Records the timestamp when a purchase order item entry is created, stored as a non-nullable datetime value.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":246,"null_count":0,"data_range":{"min":"2026-03-12 15:44:18.668789","max":"2026-03-12 15:45:45.174099"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: purchase_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column in the `purchase_order_items` table stores the non-nullable timestamp of the most recent update to a purchase order item record.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":246,"null_count":0,"data_range":{"min":"2026-03-12 15:44:18.668794","max":"2026-03-12 15:45:45.174104"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: purchase_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"ordered_qty_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"The `ordered_qty_value` column stores the numeric quantity value (up to two decimal places) of items ordered in a purchase order, which can be null.","glossary_terms":[],"cardinality":0,"null_count":246,"data_category":"continuous","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: ordered_qty","type hint: numeric(10,2)","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"ordered_qty"},{"name":"ordered_qty_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Ordered quantity unit (ea/box).","glossary_terms":[],"cardinality":0,"null_count":246,"data_category":"nominal","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: ordered_qty_unit","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity"],"concept_sources":["name","profile","values"],"concept_alias_group":"ordered_qty_unit"}],"table_description":"Line items with order quantities and explicit unit labels.","glossary_terms":[],"primary_keys":["po_item_id"],"foreign_keys":[{"column":"po_id","references":"purchase_orders.po_id"},{"column":"product_id","references":"products.product_id"}],"row_count":246,"field_classifications":{"quantity":"quantity","unit_cost":"pricing","created_at":"temporal","updated_at":"temporal","ordered_qty_value":"quantity","ordered_qty_unit":"quantity"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"po_id","target_table":"purchase_orders","target_column":"po_id","confidence":"high"},{"column":"product_id","target_table":"products","target_column":"product_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":9,"mixed_unit_groups":[],"unknown_unit_columns":["ordered_qty_unit","ordered_qty_value","quantity"]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":246,"row_count_projection_2y":246,"row_count_projection_5y":246,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"finance.currency_amount":1,"identifier.foreign_key":3,"measure.quantity":3,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-</t>
+          <t>emental":true,"column_description":"Tracks the timestamp of the most recent update to an inventory record, ensuring accurate change history.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":89,"null_count":0,"data_range":{"min":"2024-03-14 15:38:57.201565","max":"2026-03-07 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: inventory"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"stock_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"Represents the monetary value of inventory stock, stored as a numeric value with two decimal places, and may be null.","glossary_terms":["RetailDomainGlossary.Inventory"],"cardinality":0,"null_count":100,"data_category":"continuous","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.0,"concept_evidence":["type hint: numeric(10,2)","ambiguous runner-up concept"],"concept_sources":["type"],"concept_alias_group":null},{"name":"stock_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Current stock unit label.","glossary_terms":["RetailDomainGlossary.UnitOfMeasure"],"cardinality":0,"null_count":100,"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.15,"concept_evidence":["value pattern: quantity","ambiguous runner-up concept"],"concept_sources":["values"],"concept_alias_group":null}],"table_description":"Current stock levels with normalized stock unit representation.","glossary_terms":["RetailDomainGlossary.Inventory","RetailDomainGlossary.InventoryByProductAndLocation"],"primary_keys":["inventory_id"],"foreign_keys":[{"column":"product_id","references":"products.product_id"},{"column":"store_id","references":"stores.store_id"}],"row_count":100,"field_classifications":{"quantity_on_hand":"quantity","last_restocked_at":"temporal","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"product_id","target_table":"products","target_column":"product_id","confidence":"high"},{"column":"store_id","target_table":"stores","target_column":"store_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":10,"mixed_unit_groups":[],"unknown_unit_columns":["quantity_on_hand"]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":146,"row_count_projection_2y":193,"row_count_projection_5y":334,"partition_columns_candidates":["last_restocked_at","created_at","updated_at"],"classification_summary":{"concept_counts":{"identifier.foreign_key":3,"measure.quantity":1,"temporal.created_at":1,"temporal.event_time":1,"temporal.updated_at":1},"low_confidence_columns":["reorder_level","stock_unit"]},"data_quality":{"findings":[{"column":"last_restocked_at","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 100 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 3 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"last_restocked_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":3},{"column":"quantity_on_hand","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."}]}},{"table":"products","schema":"dbo","columns":[{"name":"product_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each product in the retail system, serving as the primary key for the products table.","glossary_terms":["RetailDomainGlossary.Barcode"],"cardinality":50,"null_count":0,"data_range":{"min":"156","max":"205"},"data_category":"discrete","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"supplier_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"The `supplier_id` column in the `products` table is a non-nullable foreign key referencing the `supplier_id` column in the `suppliers` table, identifying the supplier associated with each product.","glossary_terms":["RetailDomainGlossary.SupplierCode"],"cardinality":10,"null_count":0,"data_range":{"min":"33","max":"42"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"sku","type":"nvarchar(450)","nullable":false,"is_incremental":false,"column_description":"Unique alphanumeric identifier for a product used for inventory and sales tracking.","glossary_terms":["RetailDomainGlossary.Product"],"cardinality":50,"null_count":0,"data_range":{"min":"SKU-0001","max":"SKU-0050"},"data_category":"nominal","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.product_code","concept_confidence":0.7,"concept_evidence":["name token: sku","type hint: nvarchar(450)","semantic class hint: product_identifier"],"concept_sources":["name","profile","type"],"concept_alias_group":"sku"},{"name":"name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Stores the name of the product as a non-null, case-insensitive Unicode string.","glossary_terms":[],"cardinality":50,"null_count":0,"data_range":{"min":"Product 1","max":"Product 9"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"name"},{"name":"category","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Indicates the product's category classification, such as \"Books,\" \"Clothing,\" or \"Electronics,\" stored as a non-nullable nvarchar value.","glossary_terms":["RetailDomainGlossary.ProductCategory"],"cardinality":5,"null_count":0,"data_range":{"min":"Books","max":"Sports"},"data_category":"nominal","semantic_class":"category","unit_context":null,"concept_id":"entity.category","concept_confidence":0.8,"concept_evidence":["name token: category","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: categorical","profile heuristic matched"],"concept_sources":["name","profile","type"],"concept_alias_group":"category"},{"name":"unit_price","type":"numeric(10,2)","nullable":false,"is_incremental":false,"column_description":"The `unit_price` column stores the non-null selling price of a product as a numeric value with up to 10 digits and 2 decimal places, representing a currency amount.","glossary_terms":["RetailDomainGlossary.SellingPrice"],"cardinality":50,"null_count":0,"data_range":{"min":"11.09","max":"490.43"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: price","type hint: numeric(10,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"price"},{"name":"cost_price","type":"numeric(10,2)","nullable":false,"is_incremental":false,"column_description":"The `cost_price` column stores the non-null numeric cost amount (up to 10 digits with 2 decimal places) representing the purchase price of a product in the retail system.","glossary_terms":["RetailDomainGlossary.CostPrice"],"cardinality":50,"null_count":0,"data_range":{"min":"5.55","max":"358.59"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: price","type hint: numeric(10,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"price"},{"name":"active","type":"bit","nullable":false,"is_incremental":false,"column_description":"Indicates whether a product is active and available for transactions, stored as a non-nullable boolean value.","glossary_terms":[],"cardinality":1,"null_count":0,"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.0,"concept_evidence":["profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile"],"concept_alias_group":null},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column stores the non-nullable timestamp indicating when a product record was initially created in the system.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":50,"null_count":0,"data_range":{"min":"2021-03-20 15:38:57.201565","max":"2024-12-25 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: products"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column stores the non-nullable timestamp of the most recent update to a product record in the `products` table.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":50,"null_count":0,"data_range":{"min":"2021-03-20 15:38:57.201565","max":"2024-12-25 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: products"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"weight_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Source weight unit (kg/lb) used for unit inference testing.","glossary_terms":["RetailDomainGlossary.UnitOfMeasure"],"cardinality":0,"null_count":50,"data_category":"nominal","semantic_class":"mass","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":null,"concept_confidence":0.15,"concept_evidence":["value pattern: quantity","ambiguous runner-up concept"],"concept_sources":["values"],"concept_alias_group":null},{"name":"weight_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"The `weight_value` column stores the weight of a product as a numeric value with up to 10 digits and 2 decimal places, and it is nullable.","glossary_terms":["RetailDomainGlossary.UnitOfMeasure"],"cardinality":0,"null_count":50,"data_category":"continuous","semantic_class":"mass","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":null,"concept_confidence":0.0,"concept_evidence":["type hint: numeric(10,2)","ambiguous runner-up concept"],"concept_sources":["type"],"concept_alias_group":null},{"name":"length_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"Represents the length measurement of a product in numeric format, allowing null values.","glossary_terms":[],"cardinality":0,"null_count":50,"data_category":"continuous","semantic_class":"length","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":null,"concept_confidence":0.0,"concept_evidence":["type hint: numeric(10,2)","ambiguous runner-up concept"],"concept_sources":["type"],"concept_alias_group":null},{"name":"length_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Source length unit (cm/in) used for unit inference testing.","glossary_terms":["RetailDomainGlossary.UnitOfMeasure"],"cardinality":0,"null_count":50,"data_category":"nominal","semantic_class":"length","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":null,"concept_confidence":0.15,"concept_evidence":["value pattern: quantity","ambiguous runner-up concept"],"concept_sources":["values"],"concept_alias_group":null},{"name":"product_description","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"Stores optional textual details about a product, such as features or specifications.","glossary_terms":["RetailDomainGlossary.Product"],"cardinality":0,"null_count":50,"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"primary_supplier_id","type":"bigint","nullable":true,"is_incremental":false,"column_description":"Primary supplier relationship used for join candidate detection.","glossary_terms":["RetailDomainGlossary.SupplierPurchaseRelationship"],"cardinality":10,"null_count":0,"data_range":{"min":"33","max":"42"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"}],"table_description":"Master product catalog including physical units for analyzer unit-context testing.","glossary_terms":["RetailDomainGlossary.Inventory","RetailDomainGlossary.SupplierCode"],"primary_keys":["product_id"],"foreign_keys":[{"column":"primary_supplier_id","references":"suppliers.supplier_id"},{"column":"supplier_id","references":"suppliers.supplier_id"}],"row_count":50,"field_classifications":{"category":"categorical","unit_price":"pricing","cost_price":"pricing","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"primary_supplier_id","target_table":"suppliers","target_column":"supplier_id","confidence":"high"},{"column":"supplier_id","target_table":"suppliers","target_column":"supplier_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":16,"mixed_unit_groups":[],"unknown_unit_columns":["length_unit","length_value","weight_unit","weight_value"]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":68,"row_count_projection_2y":86,"row_count_projection_5y":141,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.person_name":1,"entity.category":1,"finance.currency_amount":2,"identifier.foreign_key":3,"identifier.product_code":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":["length_unit","name","product_description","weight_unit"]},"data_quality":{"findings":[{"column":"category","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 5 distinct value(s) ('Books', 'Clothing', 'Electronics', 'Home', 'Sports') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Books","Clothing","Electronics","Home","Sports"],"cardinality":5},{"column":"primary_supplier_id","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 50 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":"active","check":"delete_management","severity":"info","detail":"Active-flag column 'active' (boolean) detected \u2014 rows with active=false are logically deleted. Current distribution: True=50.","recommendation":"Filter on \"active\" = true for current records during ingestion.","delete_strategy":"soft_delete","soft_delete_column":"active","soft_delete_type":"active_flag","has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2},{"column":"weight_unit","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'mass' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"weight_value","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'mass' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"length_value","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'length' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"length_unit","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'length' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."}]}},{"table":"purchase_order_items","schema":"dbo","columns":[{"name":"po_item_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each purchase order item record in the `purchase_order_items` table.","glossary_terms":["RetailDomainGlossary.OrderLine"],"cardinality":246,"null_count":0,"data_range":{"min":"268","max":"513"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"po_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Represents the unique identifier of the associated purchase order, linking purchase order items to their parent purchase order in the `purchase_orders` table.","glossary_terms":["RetailDomainGlossary.PurchaseOrder"],"cardinality":125,"null_count":0,"data_range":{"min":"128","max":"252"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"product_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifier linking each purchase order item to a specific product in the products table.","glossary_terms":["RetailDomainGlossary.ProductCategory"],"cardinality":49,"null_count":0,"data_range":{"min":"156","max":"205"},"data_category":"discrete","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"quantity","type":"integer","nullable":false,"is_incremental":false,"column_description":"The `quantity` column in the `purchase_order_items` table stores the non-null integer value representing the number of units of a product included in a specific purchase order item.","glossary_terms":["RetailDomainGlossary.UnitOfMeasure"],"cardinality":41,"null_count":0,"data_range":{"min":"10","max":"50"},"data_category":"discrete","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: quantity","type hint: integer","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"quantity"},{"name":"unit_cost","type":"numeric(10,2)","nullable":false,"is_incremental":false,"column_description":"Represents the per-unit cost of a product in a purchase order, stored as a non-null numeric value with up to 10 digits and 2 decimal places.","glossary_terms":["RetailDomainGlossary.CostPrice"],"cardinality":49,"null_count":0,"data_range":{"min":"5.55","max":"358.59"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: unit_cost","type hint: numeric(10,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount","table context: purchase_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"unit_cost"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the non-nullable timestamp indicating when each purchase order item record was created.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":246,"null_count":0,"data_range":{"min":"2026-03-12 15:44:18.668789","max":"2026-03-12 15:45:45.174099"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: purchase_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"Records the timestamp of the most recent update to a purchase order item, ensuring accurate tracking of modifications.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":246,"null_count":0,"data_range":{"min":"2026-03-12 15:44:18.668794","max":"2026-03-12 15:45:45.174104"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: purchase_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"ordered_qty_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"The `ordered_qty_value` column stores the numeric quantity value (up to two decimal places) of items ordered in a purchase order, which can be null.","glossary_terms":["RetailDomainGlossary.PurchaseOrder"],"cardinality":0,"null_count":246,"data_category":"continuous","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: ordered_qty","type hint: numeric(10,2)","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"ordered_qty"},{"name":"ordered_qty_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Ordered quantity unit (ea/box).","glossary_terms":["RetailDomainGlossary.UnitOfMeasure"],"cardinality":0,"null_count":246,"data_category":"nominal","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: ordered_qty_unit","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity"],"concept_sources":["name","profile","values"],"concept_alias_group":"ordered_qty_unit"}],"table_description":"Line items with order quantities and explicit unit labels.","glossary_terms":["RetailDomainGlossary.OrderLine","RetailDomainGlossary.UnitOfMeasure","RetailDomainGlossary.CostPrice","RetailDomainGlossary.PurchaseOrder"],"primary_keys":["po_item_id"],"foreign_keys":[{"column":"po_id","references":"purchase_orders.po_id"},{"column":"product_id","references":"products.product_id"}],"row_count":246,"field_classifications":{"quantity":"quantity","unit_cost":"pricing","created_at":"temporal","updated_at":"temporal","ordered_qty_value":"quantity","ordered_qty_unit":"quantity"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"po_id","target_table":"purchase_orders","target_column":"po_id","confidence":"high"},{"column":"product_id","target_table":"products","target_column":"product_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":9,"mixed_unit_groups":[],"unknown_unit_columns":["ordered_qty_unit","ordered_qty_value","quantity"]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitiv</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10442,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2},{"column":"quantity","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"ordered_qty_value","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"ordered_qty_unit","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."}]}},{"table":"purchase_orders","schema":"dbo","columns":[{"name":"po_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for purchase orders in the retail operations system.","glossary_terms":[],"cardinality":125,"null_count":0,"data_range":{"min":"128","max":"252"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"supplier_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"References the unique identifier of the supplier associated with a purchase order, linking to the `suppliers.supplier_id` column.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"33","max":"42"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifies the store associated with the purchase order, referencing the `store_id` column in the `stores` table.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"status","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Indicates the current state of a purchase order, such as 'Ordered' or 'Received', using predefined category values.","glossary_terms":[],"cardinality":3,"null_count":0,"data_range":{"min":"Ordered","max":"Received"},"data_category":"nominal","semantic_class":"category","unit_context":null,"concept_id":"entity.status","concept_confidence":1.0,"concept_evidence":["name token: statu","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: categorical","value pattern: status","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"statu"},{"name":"order_date","type":"date","nullable":false,"is_incremental":false,"column_description":"The `order_date` column in the `purchase_orders` table records the date a purchase order was placed and cannot be null.","glossary_terms":[],"cardinality":123,"null_count":0,"data_range":{"min":"2021-04-09","max":"2026-03-12"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.date_only","concept_confidence":1.0,"concept_evidence":["name token: order_date","type hint: date","legacy field classification: temporal","value pattern: date_only","table context: purchase_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"order_date"},{"name":"expected_date","type":"date","nullable":true,"is_incremental":false,"column_description":"The `expected_date` column in the `purchase_orders` table records the anticipated delivery date for a purchase order, allowing null values.","glossary_terms":[],"cardinality":123,"null_count":0,"data_range":{"min":"2021-04-27","max":"2026-03-31"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.date_only","concept_confidence":1.0,"concept_evidence":["name token: expected_date","type hint: date","legacy field classification: temporal","value pattern: date_only","table context: purchase_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"expected_date"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the timestamp when a purchase order record is initially created in the system and cannot be null.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":123,"null_count":0,"data_range":{"min":"2021-04-09 15:38:57.201565","max":"2026-03-12 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: purchase_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column stores the non-null timestamp indicating the last modification date and time of a purchase order record.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":123,"null_count":0,"data_range":{"min":"2021-04-09 15:38:57.201565","max":"2026-03-12 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: purchase_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"approver_employee_id","type":"bigint","nullable":true,"is_incremental":false,"column_description":"Approver employee foreign key for procurement workflow.","glossary_terms":[],"cardinality":0,"null_count":125,"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"}],"table_description":"Procurement headers including approver employee relationship.","glossary_terms":[],"primary_keys":["po_id"],"foreign_keys":[{"column":"approver_employee_id","references":"employees.employee_id"},{"column":"store_id","references":"stores.store_id"},{"column":"supplier_id","references":"suppliers.supplier_id"}],"row_count":125,"field_classifications":{"status":"categorical","order_date":"temporal","expected_date":"temporal","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"approver_employee_id","target_table":"employees","target_column":"employee_id","confidence":"high"},{"column":"store_id","target_table":"stores","target_column":"store_id","confidence":"high"},{"column":"supplier_id","target_table":"suppliers","target_column":"supplier_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":9,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":155,"row_count_projection_2y":185,"row_count_projection_5y":276,"partition_columns_candidates":["order_date","expected_date","created_at","updated_at"],"classification_summary":{"concept_counts":{"entity.status":1,"identifier.foreign_key":4,"temporal.created_at":1,"temporal.date_only":2,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":"status","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 3 distinct value(s) ('Ordered', 'Pending', 'Received') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Ordered","Pending","Received"],"cardinality":3},{"column":"expected_date","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 125 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":"order_date","check":"late_arriving_data","severity":"info","detail":"Minor arrival delay \u2014 max lag between 'order_date' and 'created_at' is 15.7h (avg 15.7h, P95 15.7h).","recommendation":"Use 'created_at' as the watermark (preferred). If using 'order_date', add a 1\u20132 day lookback buffer.","business_date_column":"order_date","system_ts_column":"created_at","lag_stats":{"total_rows_compared":125,"min_lag_hours":15.65,"avg_lag_hours":15.65,"p95_lag_hours":15.65,"max_lag_hours":15.65,"max_lag_days":0.7,"rows_late_over_1d":0,"rows_late_over_7d":0},"recommended_lookback_days":2},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}},{"table":"sales_order_items","schema":"dbo","columns":[{"name":"sales_order_item_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for individual items within a sales order, serving as the primary key for the `sales_order_items` table.","glossary_terms":[],"cardinality":508,"null_count":0,"data_range":{"min":"497","max":"1004"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"sales_order_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifier linking each sales order item to its associated sales order in the `sales_orders` table.","glossary_terms":[],"cardinality":200,"null_count":0,"data_range":{"min":"375","max":"574"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"product_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"References the unique identifier of the product associated with a sales order item, linking to the `products.product_id` column.","glossary_terms":[],"cardinality":50,"null_count":0,"data_range":{"min":"156","max":"205"},"data_category":"discrete","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"quantity","type":"integer","nullable":false,"is_incremental":false,"column_description":"The \"quantity\" column in the \"sales_order_items\" table stores the non-null integer value representing the number of units of a product included in a specific sales order item.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"1","max":"5"},"data_category":"discrete","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: quantity","type hint: integer","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"quantity"},{"name":"unit_price","type":"numeric(15,2)","nullable":false,"is_incremental":false,"column_description":"Represents the per-unit price of a product in a sales order item, stored as a non-null numeric value with up to 15 digits and 2 decimal places.","glossary_terms":[],"cardinality":50,"null_count":0,"data_range":{"min":"11.09","max":"490.43"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: price","type hint: numeric(15,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount","table context: sales_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"price"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column in the `sales_order_items` table stores the non-nullable timestamp indicating when a sales order item record was created.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":508,"null_count":0,"data_range":{"min":"2026-03-12 15:41:01.155388","max":"2026-03-12 15:43:38.264437"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: sales_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column stores the non-nullable timestamp of the most recent update to a sales order item record for tracking modification history.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":508,"null_count":0,"data_range":{"min":"2026-03-12 15:41:01.155390","max":"2026-03-12 15:43:38.264447"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: sales_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"sold_qty_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"Represents the numeric value of the quantity sold for a sales order item, allowing up to two decimal places and nullable for cases where the quantity is not recorded.","glossary_terms":[],"cardinality":0,"null_count":508,"data_category":"continuous","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: sold_qty","type hint: numeric(10,2)","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"sold_qty"},{"name":"sold_qty_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Sold quantity unit (ea/box).","glossary_terms":[],"cardinality":0,"null_count":508,"data_category":"nominal","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: sold_qty_unit","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity"],"concept_sources":["name","profile","values"],"concept_alias_group":"sold_qty_unit"}],"table_description":"Sales line items with sold quantity and explicit unit labels.","glossary_terms":[],"primary_keys":["sales_order_item_id"],"foreign_keys":[{"column":"product_id","references":"products.product_id"},{"column":"sales_order_id","references":"sales_orders.sales_order_id"}],"row_count":508,"field_classifications":{"quantity":"quantity","unit_price":"pricing","created_at":"temporal","updated_at":"temporal","sold_qty_value":"quantity","sold_qty_unit":"quantity"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"product_id","target_table":"products","target_column":"product_id","confidence":"high"},{"column":"sales_order_id","target_table":"sales_orders","target_column":"sales_order_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":9,"mixed_unit_groups":[],"unknown_unit_columns":["quantity","sold_qty_unit","sold_qty_value"]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":508,"row_count_projection_2y":508,"row_count_projection_5y":508,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"finance.currency_amount":1,"identifier.foreign_key":3,"measure.quantity":3,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2},{"column":"quantity","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"sold_qty_value","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"sold_qty_unit","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."}]}},{"table":"sales_orders","schema":"dbo","columns":[{"name":"sales_order_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each sales order in the system.","glossary_terms":[],"cardinality":200,"null_count":0,"data_range":{"min":"375","max":"574"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifies the store associated with a sales order, referencing the `store_id` column in the `stores` table.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"customer_id","type":"bigint","nullable":true,"is_incremental":false,"column_description":"Identifies the customer associated with a sales order, referencing the `customer_id` column in the `customers` table; nullable to accommodate orders without a registered customer.","glossary_terms":[],"cardinality":76,"null_count":0,"data_range":{"min":"404","max":"502"},"data_category":"discrete","semantic_class":"customer_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"employee_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifies the employee responsible for processing the sales order, referencing the `employees.employee_id` column.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"64","max":"83"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"order_date","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `order_date` column records the date and time when a sales order was placed, stored as a non-nullable `datetime2` value.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":191,"null_count":0,"data_range":{"min":"2021-03-14 15:38:57.201565","max":"2026-03-11 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.date_only","concept_confidence":0.9,"concept_evidence":["name token: order_date","type hint: datetime2","legacy field classification: temporal","table context: sales_orders","cross-table consensus: 2 similar columns"],"concept_sources":["cross_table_consensus","name","profile","table_context","type"],"concept_alias_group":"order_date"},{"name":"status","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Indicates the current state of a sales order, such as 'Pending' or 'Completed', stored as a non-nullable text category.","glossary_terms":[],"cardinality":3,"null_count":0,"data_range":{"min":"Completed","max":"Shipped"},"data_category":"nominal","semantic_class":"category","unit_context":null,"concept_id":"entity.status","concept_confidence":1.0,"concept_evidence":["name token: statu","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: categorical","value pattern: status","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"statu"},{"name":"total_amount","type":"numeric(12,2)","nullable":false,"is_incremental":false,"column_description":"The `total_amount` column in the `sales_orders` table stores the non-nullable total monetary value of a sales order as a numeric value with up to 12 digits and 2 decimal places.","glossary_terms":[],"cardinality":200,"null_count":0,"data_range":{"min":"66.47","max":"998.76"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: amount","type hint: numeric(12,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount","table context: sales_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"amount"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the timestamp when a sales order entry was initially created, stored as a non-nullable `datetime2` value.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":191,"null_count":0,"data_range":{"min":"2021-03-14 15:38:57.201565","max":"2026-03-11 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: sales_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column records the timestamp of the most recent update to a sales order, ensuring accurate tracking of modifications, and it is mandatory.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":191,"null_count":0,"data_range":{"min":"2021-03-14 15:38:57.201565","max":"2026-03-11 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: sales_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"sales_rep_employee_id","type":"bigint","nullable":true,"is_incremental":false,"column_description":"Sales representative foreign key for order ownership.","glossary_terms":[],"cardinality":0,"null_count":200,"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"}],"table_description":"Sales headers including assigned sales representative relationship.","glossary_terms":</t>
+          <t>e_fields":false,"row_count_projection_1y":246,"row_count_projection_2y":246,"row_count_projection_5y":246,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"finance.currency_amount":1,"identifier.foreign_key":3,"measure.quantity":3,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2},{"column":"quantity","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"ordered_qty_value","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"ordered_qty_unit","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."}]}},{"table":"purchase_orders","schema":"dbo","columns":[{"name":"po_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for purchase orders in the system.","glossary_terms":["RetailDomainGlossary.PurchaseOrder"],"cardinality":125,"null_count":0,"data_range":{"min":"128","max":"252"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"supplier_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifies the supplier associated with a purchase order, referencing the `supplier_id` column in the `suppliers` table.","glossary_terms":["RetailDomainGlossary.SupplierCode"],"cardinality":10,"null_count":0,"data_range":{"min":"33","max":"42"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifies the store associated with the purchase order, referencing the `store_id` column in the `stores` table.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"status","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Indicates the current state of a purchase order (e.g., \"Ordered,\" \"Received\") as a non-null categorical value.","glossary_terms":["RetailDomainGlossary.OrderStatus"],"cardinality":3,"null_count":0,"data_range":{"min":"Ordered","max":"Received"},"data_category":"nominal","semantic_class":"category","unit_context":null,"concept_id":"entity.status","concept_confidence":1.0,"concept_evidence":["name token: statu","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: categorical","value pattern: status","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"statu"},{"name":"order_date","type":"date","nullable":false,"is_incremental":false,"column_description":"The `order_date` column in the `purchase_orders` table records the date a purchase order was placed, is mandatory, and uses the `date` data type.","glossary_terms":[],"cardinality":123,"null_count":0,"data_range":{"min":"2021-04-09","max":"2026-03-12"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.date_only","concept_confidence":1.0,"concept_evidence":["name token: order_date","type hint: date","legacy field classification: temporal","value pattern: date_only","table context: purchase_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"order_date"},{"name":"expected_date","type":"date","nullable":true,"is_incremental":false,"column_description":"The `expected_date` column in the `purchase_orders` table records the anticipated delivery date for a purchase order, allowing null values.","glossary_terms":["RetailDomainGlossary.OrderDeliveryRelationship"],"cardinality":123,"null_count":0,"data_range":{"min":"2021-04-27","max":"2026-03-31"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.date_only","concept_confidence":1.0,"concept_evidence":["name token: expected_date","type hint: date","legacy field classification: temporal","value pattern: date_only","table context: purchase_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"expected_date"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column stores the non-nullable timestamp indicating when a purchase order record was initially created in the system.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":123,"null_count":0,"data_range":{"min":"2021-04-09 15:38:57.201565","max":"2026-03-12 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: purchase_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column stores the non-nullable timestamp of the most recent update to a purchase order record.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":123,"null_count":0,"data_range":{"min":"2021-04-09 15:38:57.201565","max":"2026-03-12 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: purchase_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"approver_employee_id","type":"bigint","nullable":true,"is_incremental":false,"column_description":"Approver employee foreign key for procurement workflow.","glossary_terms":[],"cardinality":0,"null_count":125,"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"}],"table_description":"Procurement headers including approver employee relationship.","glossary_terms":["RetailDomainGlossary.PurchaseOrder","RetailDomainGlossary.OrderStatus"],"primary_keys":["po_id"],"foreign_keys":[{"column":"approver_employee_id","references":"employees.employee_id"},{"column":"store_id","references":"stores.store_id"},{"column":"supplier_id","references":"suppliers.supplier_id"}],"row_count":125,"field_classifications":{"status":"categorical","order_date":"temporal","expected_date":"temporal","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"approver_employee_id","target_table":"employees","target_column":"employee_id","confidence":"high"},{"column":"store_id","target_table":"stores","target_column":"store_id","confidence":"high"},{"column":"supplier_id","target_table":"suppliers","target_column":"supplier_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":9,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":155,"row_count_projection_2y":185,"row_count_projection_5y":276,"partition_columns_candidates":["order_date","expected_date","created_at","updated_at"],"classification_summary":{"concept_counts":{"entity.status":1,"identifier.foreign_key":4,"temporal.created_at":1,"temporal.date_only":2,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":"status","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 3 distinct value(s) ('Ordered', 'Pending', 'Received') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Ordered","Pending","Received"],"cardinality":3},{"column":"expected_date","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 125 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":"order_date","check":"late_arriving_data","severity":"info","detail":"Minor arrival delay \u2014 max lag between 'order_date' and 'created_at' is 15.7h (avg 15.7h, P95 15.7h).","recommendation":"Use 'created_at' as the watermark (preferred). If using 'order_date', add a 1\u20132 day lookback buffer.","business_date_column":"order_date","system_ts_column":"created_at","lag_stats":{"total_rows_compared":125,"min_lag_hours":15.65,"avg_lag_hours":15.65,"p95_lag_hours":15.65,"max_lag_hours":15.65,"max_lag_days":0.7,"rows_late_over_1d":0,"rows_late_over_7d":0},"recommended_lookback_days":2},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}},{"table":"sales_order_items","schema":"dbo","columns":[{"name":"sales_order_item_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each sales order item in the sales_order_items table.","glossary_terms":["RetailDomainGlossary.OrderLine"],"cardinality":508,"null_count":0,"data_range":{"min":"497","max":"1004"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"sales_order_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifier linking each sales order item to its associated sales order in the `sales_orders` table.","glossary_terms":["RetailDomainGlossary.SalesOrder"],"cardinality":200,"null_count":0,"data_range":{"min":"375","max":"574"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"product_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifier for the product associated with the sales order item, referencing the primary key in the products table.","glossary_terms":["RetailDomainGlossary.ProductCategory"],"cardinality":50,"null_count":0,"data_range":{"min":"156","max":"205"},"data_category":"discrete","semantic_class":"product_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"quantity","type":"integer","nullable":false,"is_incremental":false,"column_description":"The \"quantity\" column in the \"sales_order_items\" table stores the number of units of a product included in a sales order item, represented as a non-null integer.","glossary_terms":["RetailDomainGlossary.OrderLine"],"cardinality":5,"null_count":0,"data_range":{"min":"1","max":"5"},"data_category":"discrete","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: quantity","type hint: integer","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"quantity"},{"name":"unit_price","type":"numeric(15,2)","nullable":false,"is_incremental":false,"column_description":"The `unit_price` column in the `sales_order_items` table stores the per-unit selling price of a product in the sales order as a non-null numeric value with two decimal places.","glossary_terms":["RetailDomainGlossary.SellingPrice"],"cardinality":50,"null_count":0,"data_range":{"min":"11.09","max":"490.43"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: price","type hint: numeric(15,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount","table context: sales_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"price"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"Records the timestamp when a sales order item entry is created, ensuring accurate tracking of creation events.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":508,"null_count":0,"data_range":{"min":"2026-03-12 15:41:01.155388","max":"2026-03-12 15:43:38.264437"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: sales_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column in the `sales_order_items` table stores the non-nullable timestamp of the most recent update to a sales order item record.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":508,"null_count":0,"data_range":{"min":"2026-03-12 15:41:01.155390","max":"2026-03-12 15:43:38.264447"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: sales_order_items"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"sold_qty_value","type":"numeric(10,2)","nullable":true,"is_incremental":false,"column_description":"The `sold_qty_value` column stores the numeric value representing the quantity of a product sold in a sales order item, allowing up to two decimal places, and can be null.","glossary_terms":["RetailDomainGlossary.OrderLine"],"cardinality":0,"null_count":508,"data_category":"continuous","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: sold_qty","type hint: numeric(10,2)","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"sold_qty"},{"name":"sold_qty_unit","type":"nvarchar(16)","nullable":true,"is_incremental":false,"column_description":"Sold quantity unit (ea/box).","glossary_terms":["RetailDomainGlossary.UnitOfMeasure"],"cardinality":0,"null_count":508,"data_category":"nominal","semantic_class":"quantity","unit_context":{"detected_unit":null,"canonical_unit":null,"unit_system":"unknown","conversion":null,"detection_confidence":"low","detection_source":"combined","notes":"Semantic class suggests units, but no explicit source unit token was detected."},"concept_id":"measure.quantity","concept_confidence":1.0,"concept_evidence":["name token: sold_qty_unit","legacy field classification: quantity","semantic class hint: quantity","value pattern: quantity"],"concept_sources":["name","profile","values"],"concept_alias_group":"sold_qty_unit"}],"table_description":"Sales line items with sold quantity and explicit unit labels.","glossary_terms":["RetailDomainGlossary.OrderLine","RetailDomainGlossary.SalesOrder","RetailDomainGlossary.UnitOfMeasure"],"primary_keys":["sales_order_item_id"],"foreign_keys":[{"column":"product_id","references":"products.product_id"},{"column":"sales_order_id","references":"sales_orders.sales_order_id"}],"row_count":508,"field_classifications":{"quantity":"quantity","unit_price":"pricing","created_at":"temporal","updated_at":"temporal","sold_qty_value":"quantity","sold_qty_unit":"quantity"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"product_id","target_table":"products","target_column":"product_id","confidence":"high"},{"column":"sales_order_id","target_table":"sales_orders","target_column":"sales_order_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":9,"mixed_unit_groups":[],"unknown_unit_columns":["quantity","sold_qty_unit","sold_qty_value"]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":508,"row_count_projection_2y":508,"row_count_projection_5y":508,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"finance.currency_amount":1,"identifier.foreign_key":3,"measure.quantity":3,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2},{"column":"quantity","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"sold_qty_value","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."},{"column":"sold_qty_unit","check":"unit_unknown","severity":"warning","detail":"Column semantic class 'quantity' has unknown source units.","recommendation":"Add explicit source unit mapping for this field to enable safe aggregation."}]}},{"table":"sales_orders","schema":"dbo","columns":[{"name":"sales_order_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each sales order in the system, serving as the primary key for the sales_orders table.","glossary_terms":["RetailDomainGlossary.SalesOrder"],"cardinality":200,"null_count":0,"data_range":{"min":"375","max":"574"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Identifies the store associated with a sales order, referencing the `store_id` column in the `stores` table.","glossary_terms":["RetailDomainGlossary.SalesChannel"],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"customer_id","type":"bigint","nullable":true,"is_incremental":false,"column_description":"Represents the identifier of the customer associated with a sales order, referencing the `customer_id` column in the `customers` table, and may be null if no customer is linked.","glossary_terms":["RetailDomainGlossary.CustomerIdentifier"],"cardinality":76,"null_count":0,"data_range":{"min":"404","max":"502"},"data_category":"discrete","semantic_class":"customer_identifier","unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"employee_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Represents the unique identifier of the employee associated with the sales order, referencing the `employees.employee_id` column.","glossary_terms":[],"cardinality":20,"null_count":0,"data_range":{"min":"64","max":"83"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"},{"name":"order_date","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `order_date` column records the date and time when a sales order was placed, stored as a non-nullable `datetime2` value.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":191,"null_count":0,"data_range":{"min":"2021-03-14 15:38:57.201565","max":"2026-03-11 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.date_only","concept_confidence":0.9,"concept_evidence":["name token: order_date","type hint: datetime2","legacy field classification: temporal","table context: sales_orders","cross-table consensus: 2 similar columns"],"concept_sources":["cross_table_consensus","name","profile","table_context","type"],"concept_alias_group":"order_date"},{"name":"status","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"Indicates the current state of a sales order, such as 'Pending' or 'Completed', stored as a non-nullable text category.","glossary_terms":["RetailDomainGlossary.OrderStatus"],"cardinality":3,"null_count":0,"data_range":{"min":"Completed","max":"Shipped"},"data_category":"nominal","semantic_class":"category","unit_context":null,"concept_id":"entity.status","concept_confidence":1.0,"concept_evidence":["name token: statu","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: categorical","value pattern: status","profile heuristic matched"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"statu"},{"name":"total_amount","type":"numeric(12,2)","nullable":false,"is_incremental":false,"column_description":"The `total_amount` column in the `sales_orders` table stores the non-nullable total monetary value of a sales order as a numeric value with up to 12 digits and 2 decimal places.","glossary_terms":["RetailDomainGlossary.SalesOrder"],"cardinality":200,"null_count":0,"data_range":{"min":"66.47","max":"998.76"},"data_category":"continuous","semantic_class":"currency_amount","unit_context":null,"concept_id":"finance.currency_amount","concept_confidence":1.0,"concept_evidence":["name token: amount","type hint: numeric(12,2)","legacy field classification: pricing","semantic class hint: currency_amount","value pattern: currency_amount","table context: sales_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"amount"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the timestamp when a sales order record is initially created, stored as a non-nullable `datetime2` value.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardina</t>
         </is>
       </c>
     </row>
@@ -10356,7 +10452,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[],"primary_keys":["sales_order_id"],"foreign_keys":[{"column":"customer_id","references":"customers.customer_id"},{"column":"employee_id","references":"employees.employee_id"},{"column":"sales_rep_employee_id","references":"employees.employee_id"},{"column":"store_id","references":"stores.store_id"}],"row_count":200,"field_classifications":{"customer_id":"identifier","order_date":"temporal","status":"categorical","total_amount":"pricing","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"customer_id","target_table":"customers","target_column":"customer_id","confidence":"high"},{"column":"employee_id","target_table":"employees","target_column":"employee_id","confidence":"high"},{"column":"sales_rep_employee_id","target_table":"employees","target_column":"employee_id","confidence":"high"},{"column":"store_id","target_table":"stores","target_column":"store_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":10,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":242,"row_count_projection_2y":284,"row_count_projection_5y":412,"partition_columns_candidates":["order_date","created_at","updated_at"],"classification_summary":{"concept_counts":{"entity.status":1,"finance.currency_amount":1,"identifier.foreign_key":5,"temporal.created_at":1,"temporal.date_only":1,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":"status","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 3 distinct value(s) ('Completed', 'Pending', 'Shipped') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Completed","Pending","Shipped"],"cardinality":3},{"column":"customer_id","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 200 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":"order_date","check":"late_arriving_data","severity":"info","detail":"Data arrives promptly \u2014 max lag between 'order_date' and 'created_at' is 0.0h. Standard watermarking on 'created_at' is safe.","recommendation":"Use 'created_at' as the incremental watermark. No special lookback window needed.","business_date_column":"order_date","system_ts_column":"created_at","lag_stats":{"total_rows_compared":200,"min_lag_hours":0.0,"avg_lag_hours":0.0,"p95_lag_hours":0.0,"max_lag_hours":0.0,"max_lag_days":0.0,"rows_late_over_1d":0,"rows_late_over_7d":0},"recommended_lookback_days":1},{"column":null,"check":"timezone","severity":"info","detail":"All 3 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"order_date","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":3}]}},{"table":"stores","schema":"dbo","columns":[{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each store in the retail operations system.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"The \"name\" column in the \"stores\" table is a non-nullable nvarchar field storing the name of each retail store.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"Airport Shop","max":"Suburb Store"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"name"},{"name":"code","type":"nvarchar(450)","nullable":false,"is_incremental":false,"column_description":"Unique identifier for a store, typically represented as an alphanumeric code.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"AIR","max":"SUB"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: nvarchar(450)","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"address","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"address\" column in the \"stores\" table stores the street address of a retail store location as a nullable Unicode string.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"1 Main St","max":"5 Main St"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.address","concept_confidence":0.55,"concept_evidence":["name token: address","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"address"},{"name":"city","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"city\" column in the \"stores\" table stores the name of the city where a store is located, allowing null values.","glossary_terms":[],"cardinality":3,"null_count":0,"data_range":{"min":"Cork","max":"Limerick"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"state","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"Indicates the state or province where the store is located, stored as a nullable text field.","glossary_terms":[],"cardinality":3,"null_count":0,"data_range":{"min":"Connacht","max":"Munster"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"postal_code","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"postal_code\" column in the \"stores\" table stores the postal or ZIP code of a store location as a nullable, case-insensitive string.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"10000","max":"10004"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.address","concept_confidence":0.55,"concept_evidence":["name token: postal_code","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"postal_code"},{"name":"phone","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"Stores.phone is an optional nvarchar column storing the contact phone number for a store location.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"555-3000","max":"555-3004"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.phone","concept_confidence":1.0,"concept_evidence":["name token: phone","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: contact","value pattern: phone","sensitive hint: pii_contact"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"phone"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the non-nullable timestamp indicating when a store record was initially created in the system.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":5,"null_count":0,"data_range":{"min":"2021-07-26 15:38:57.201565","max":"2025-01-31 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: stores"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column records the timestamp of the most recent update to a store's record and cannot be null.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":5,"null_count":0,"data_range":{"min":"2021-07-26 15:38:57.201565","max":"2025-01-31 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: stores"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"}],"table_description":"The \"stores\" table contains details about retail store locations, including unique identifiers, names, addresses, contact information, and timestamps for record creation and updates.","glossary_terms":[],"primary_keys":["store_id"],"foreign_keys":[],"row_count":5,"field_classifications":{"phone":"contact","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{"address":"pii_address","postal_code":"pii_address","phone":"pii_contact"},"incremental_columns":["updated_at"],"join_candidates":[],"unit_summary":{"columns_with_units":0,"columns_without_units":10,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":false,"has_sensitive_fields":true,"row_count_projection_1y":17,"row_count_projection_2y":29,"row_count_projection_5y":65,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.address":2,"contact.person_name":1,"contact.phone":1,"identifier.foreign_key":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":["address","city","code","name","postal_code","state"]},"data_quality":{"findings":[{"column":"city","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 3 distinct value(s) ('Cork', 'Galway', 'Limerick') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Cork","Galway","Limerick"],"cardinality":3},{"column":"state","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 3 distinct value(s) ('Connacht', 'Leinster', 'Munster') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Connacht","Leinster","Munster"],"cardinality":3},{"column":"postal_code","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 5 distinct value(s) ('10000', '10001', '10002', '10003', '10004') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["10000","10001","10002","10003","10004"],"cardinality":5},{"column":"address","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"city","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"state","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"postal_code","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"phone","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}},{"table":"suppliers","schema":"dbo","columns":[{"name":"supplier_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each supplier, serving as the primary key in the suppliers table.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"33","max":"42"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"The \"name\" column in the \"suppliers\" table is a non-nullable nvarchar field intended to store the name of the supplier, though sample data indicates it is currently unused.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"Supplier 1","max":"Supplier 9"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"name"},{"name":"contact_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The `contact_name` column in the `suppliers` table stores the name of the primary contact person for a supplier, allowing null values.","glossary_terms":[],"cardinality":0,"null_count":10,"data_category":"nominal","semantic_class":"person_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: contact_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"contact_name"},{"name":"email","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"email\" column in the \"suppliers\" table stores the email address of a supplier as a nullable nvarchar value for contact purposes.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"supplier1@example.com","max":"supplier9@example.com"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.email","concept_confidence":1.0,"concept_evidence":["name token: email","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: contact","value pattern: email","sensitive hint: pii_contact"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"email"},{"name":"phone","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"phone\" column in the \"suppliers\" table stores the supplier's contact phone number as a nullable string.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"555-2001","max":"555-2010"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.phone","concept_confidence":1.0,"concept_evidence":["name token: phone","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: contact","value pattern: phone","sensitive hint: pii_contact"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"phone"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column records the non-nullable timestamp indicating when a supplier record was initially created in the system.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":10,"null_count":0,"data_range":{"min":"2021-03-22 15:38:57.201565","max":"2024-02-25 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: suppliers"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column stores the non-nullable timestamp of the most recent update to a supplier record.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":10,"null_count":0,"data_range":{"min":"2021-03-22 15:38:57.201565","max":"2024-02-25 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: suppliers"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"}],"table_description":"The \"suppliers\" table stores information about suppliers, including their unique identifier, name, contact details, and timestamps for record creation and updates.","glossary_terms":[],"primary_keys":["supplier_id"],"foreign_keys":[],"row_count":10,"field_classifications":{"contact_name":"person_name","email":"contact","phone":"contact","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{"email":"pii_contact","phone":"pii_contact"},"incremental_columns":["updated_at"],"join_candidates":[],"unit_summary":{"columns_with_units":0,"columns_without_units":7,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":false,"has_sensitive_fields":true,"row_count_projection_1y":22,"row_count_projection_2y":35,"row_count_projection_5y":74,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.email":1,"contact.person_name":2,"contact.phone":1,"identifier.foreign_key":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":["contact_name","name"]},"data_quality":{"findings":[{"column":"email","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 10 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"phone","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 10 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}}]}</t>
+          <t>lity":191,"null_count":0,"data_range":{"min":"2021-03-14 15:38:57.201565","max":"2026-03-11 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: sales_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column records the timestamp of the most recent update to a sales order, stored as a non-nullable datetime2 value.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":191,"null_count":0,"data_range":{"min":"2021-03-14 15:38:57.201565","max":"2026-03-11 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: sales_orders"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"},{"name":"sales_rep_employee_id","type":"bigint","nullable":true,"is_incremental":false,"column_description":"Sales representative foreign key for order ownership.","glossary_terms":[],"cardinality":0,"null_count":200,"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.9,"concept_evidence":["name token: id","type hint: bigint","structural hint: join candidate"],"concept_sources":["name","profile","type"],"concept_alias_group":"id"}],"table_description":"Sales headers including assigned sales representative relationship.","glossary_terms":["RetailDomainGlossary.SalesOrder","RetailDomainGlossary.CustomerIdentifier","RetailDomainGlossary.OrderStatus"],"primary_keys":["sales_order_id"],"foreign_keys":[{"column":"customer_id","references":"customers.customer_id"},{"column":"employee_id","references":"employees.employee_id"},{"column":"sales_rep_employee_id","references":"employees.employee_id"},{"column":"store_id","references":"stores.store_id"}],"row_count":200,"field_classifications":{"customer_id":"identifier","order_date":"temporal","status":"categorical","total_amount":"pricing","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{},"incremental_columns":["updated_at"],"join_candidates":[{"column":"customer_id","target_table":"customers","target_column":"customer_id","confidence":"high"},{"column":"employee_id","target_table":"employees","target_column":"employee_id","confidence":"high"},{"column":"sales_rep_employee_id","target_table":"employees","target_column":"employee_id","confidence":"high"},{"column":"store_id","target_table":"stores","target_column":"store_id","confidence":"high"}],"unit_summary":{"columns_with_units":0,"columns_without_units":10,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":true,"has_sensitive_fields":false,"row_count_projection_1y":242,"row_count_projection_2y":284,"row_count_projection_5y":412,"partition_columns_candidates":["order_date","created_at","updated_at"],"classification_summary":{"concept_counts":{"entity.status":1,"finance.currency_amount":1,"identifier.foreign_key":5,"temporal.created_at":1,"temporal.date_only":1,"temporal.updated_at":1},"low_confidence_columns":[]},"data_quality":{"findings":[{"column":"status","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 3 distinct value(s) ('Completed', 'Pending', 'Shipped') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Completed","Pending","Shipped"],"cardinality":3},{"column":"customer_id","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 200 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":"order_date","check":"late_arriving_data","severity":"info","detail":"Data arrives promptly \u2014 max lag between 'order_date' and 'created_at' is 0.0h. Standard watermarking on 'created_at' is safe.","recommendation":"Use 'created_at' as the incremental watermark. No special lookback window needed.","business_date_column":"order_date","system_ts_column":"created_at","lag_stats":{"total_rows_compared":200,"min_lag_hours":0.0,"avg_lag_hours":0.0,"p95_lag_hours":0.0,"max_lag_hours":0.0,"max_lag_days":0.0,"rows_late_over_1d":0,"rows_late_over_7d":0},"recommended_lookback_days":1},{"column":null,"check":"timezone","severity":"info","detail":"All 3 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"order_date","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":3}]}},{"table":"stores","schema":"dbo","columns":[{"name":"store_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each store in the retail operations system.","glossary_terms":["RetailDomainGlossary.StoreCode"],"cardinality":5,"null_count":0,"data_range":{"min":"19","max":"23"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"The \"name\" column in the \"stores\" table is a non-nullable nvarchar field storing the name of a retail store.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"Airport Shop","max":"Suburb Store"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"name"},{"name":"code","type":"nvarchar(450)","nullable":false,"is_incremental":false,"column_description":"Unique alphanumeric identifier for a store, used for internal reference and operations.","glossary_terms":["RetailDomainGlossary.StoreCode"],"cardinality":5,"null_count":0,"data_range":{"min":"AIR","max":"SUB"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: nvarchar(450)","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"address","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"address\" column in the \"stores\" table stores the street address of a retail store location as a nullable Unicode string.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"1 Main St","max":"5 Main St"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.address","concept_confidence":0.55,"concept_evidence":["name token: address","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"address"},{"name":"city","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"city\" column in the \"stores\" table stores the name of the city where a store is located, allowing null values.","glossary_terms":[],"cardinality":3,"null_count":0,"data_range":{"min":"Cork","max":"Limerick"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"state","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"state\" column in the \"stores\" table stores the name of the state or province where a store is located, allowing null values.","glossary_terms":[],"cardinality":3,"null_count":0,"data_range":{"min":"Connacht","max":"Munster"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":null,"concept_confidence":0.1,"concept_evidence":["type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","profile heuristic matched","ambiguous runner-up concept"],"concept_sources":["profile","type"],"concept_alias_group":null},{"name":"postal_code","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"postal_code\" column in the \"stores\" table stores the postal or ZIP code of a store location as a nullable string.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"10000","max":"10004"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.address","concept_confidence":0.55,"concept_evidence":["name token: postal_code","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"postal_code"},{"name":"phone","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"phone\" column in the \"stores\" table stores the contact phone number of a store as a nullable nvarchar value.","glossary_terms":[],"cardinality":5,"null_count":0,"data_range":{"min":"555-3000","max":"555-3004"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.phone","concept_confidence":1.0,"concept_evidence":["name token: phone","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: contact","value pattern: phone","sensitive hint: pii_contact"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"phone"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"The `created_at` column stores the non-nullable timestamp indicating when a store record was initially created in the system.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":5,"null_count":0,"data_range":{"min":"2021-07-26 15:38:57.201565","max":"2025-01-31 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: stores"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column records the timestamp of the most recent update to a store's record and cannot be null.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":5,"null_count":0,"data_range":{"min":"2021-07-26 15:38:57.201565","max":"2025-01-31 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: stores"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"}],"table_description":"The \"stores\" table stores information about retail store locations, including unique identifiers, names, codes, addresses, contact details, and timestamps for record creation and updates.","glossary_terms":["RetailDomainGlossary.StoreCode"],"primary_keys":["store_id"],"foreign_keys":[],"row_count":5,"field_classifications":{"phone":"contact","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{"address":"pii_address","postal_code":"pii_address","phone":"pii_contact"},"incremental_columns":["updated_at"],"join_candidates":[],"unit_summary":{"columns_with_units":0,"columns_without_units":10,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":false,"has_sensitive_fields":true,"row_count_projection_1y":17,"row_count_projection_2y":29,"row_count_projection_5y":65,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.address":2,"contact.person_name":1,"contact.phone":1,"identifier.foreign_key":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":["address","city","code","name","postal_code","state"]},"data_quality":{"findings":[{"column":"city","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 3 distinct value(s) ('Cork', 'Galway', 'Limerick') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Cork","Galway","Limerick"],"cardinality":3},{"column":"state","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 3 distinct value(s) ('Connacht', 'Leinster', 'Munster') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["Connacht","Leinster","Munster"],"cardinality":3},{"column":"postal_code","check":"controlled_value_candidate","severity":"warning","detail":"Text column with 5 distinct value(s) ('10000', '10001', '10002', '10003', '10004') but no CHECK, ENUM, or FK constraint","recommendation":"Add a CHECK constraint, convert to an ENUM type, or create a lookup/reference table to prevent invalid values","distinct_values":["10000","10001","10002","10003","10004"],"cardinality":5},{"column":"address","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"city","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"state","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"postal_code","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"phone","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 5 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}},{"table":"suppliers","schema":"dbo","columns":[{"name":"supplier_id","type":"bigint","nullable":false,"is_incremental":false,"column_description":"Unique identifier for each supplier, serving as the primary key in the suppliers table.","glossary_terms":["RetailDomainGlossary.SupplierCode"],"cardinality":10,"null_count":0,"data_range":{"min":"33","max":"42"},"data_category":"discrete","semantic_class":null,"unit_context":null,"concept_id":"identifier.foreign_key","concept_confidence":0.6,"concept_evidence":["name token: id","type hint: bigint","cross-table consensus: 16 similar columns","ambiguous runner-up concept"],"concept_sources":["cross_table_consensus","name","type"],"concept_alias_group":"id"},{"name":"name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":false,"is_incremental":false,"column_description":"The \"name\" column in the \"suppliers\" table is a non-nullable nvarchar field intended to store the name of the supplier, though sample data indicates it is currently unused.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"Supplier 1","max":"Supplier 9"},"data_category":"nominal","semantic_class":null,"unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"name"},{"name":"contact_name","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"Stores the name of the primary contact person for a supplier, allowing null values.","glossary_terms":[],"cardinality":0,"null_count":10,"data_category":"nominal","semantic_class":"person_name","unit_context":null,"concept_id":"contact.person_name","concept_confidence":0.55,"concept_evidence":["name token: contact_name","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\""],"concept_sources":["name","type"],"concept_alias_group":"contact_name"},{"name":"email","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"email\" column in the \"suppliers\" table stores the email address of a supplier as a nullable nvarchar value for contact purposes.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"supplier1@example.com","max":"supplier9@example.com"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.email","concept_confidence":1.0,"concept_evidence":["name token: email","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: contact","value pattern: email","sensitive hint: pii_contact"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"email"},{"name":"phone","type":"nvarchar collate \"sql_latin1_general_cp1_ci_as\"","nullable":true,"is_incremental":false,"column_description":"The \"phone\" column in the \"suppliers\" table stores the contact phone number of a supplier as a nullable string.","glossary_terms":[],"cardinality":10,"null_count":0,"data_range":{"min":"555-2001","max":"555-2010"},"data_category":"nominal","semantic_class":"contact","unit_context":null,"concept_id":"contact.phone","concept_confidence":1.0,"concept_evidence":["name token: phone","type hint: nvarchar collate \"sql_latin1_general_cp1_ci_as\"","legacy field classification: contact","value pattern: phone","sensitive hint: pii_contact"],"concept_sources":["name","profile","type","values"],"concept_alias_group":"phone"},{"name":"created_at","type":"datetime2","nullable":false,"is_incremental":false,"column_description":"Records the timestamp when a supplier entry is initially created in the system, stored as a non-nullable datetime value.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":10,"null_count":0,"data_range":{"min":"2021-03-22 15:38:57.201565","max":"2024-02-25 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.created_at","concept_confidence":1.0,"concept_evidence":["name token: created_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: suppliers"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"created_at"},{"name":"updated_at","type":"datetime2","nullable":false,"is_incremental":true,"column_description":"The `updated_at` column stores the non-nullable timestamp of the most recent update to a supplier record in the `suppliers` table.","glossary_terms":[],"column_timezone":"(UTC) Coordinated Universal Time","cardinality":10,"null_count":0,"data_range":{"min":"2021-03-22 15:38:57.201565","max":"2024-02-25 15:38:57.201565"},"data_category":"continuous","semantic_class":"timestamp","unit_context":null,"concept_id":"temporal.updated_at","concept_confidence":1.0,"concept_evidence":["name token: updated_at","type hint: datetime2","legacy field classification: temporal","value pattern: timestamp","table context: suppliers"],"concept_sources":["name","profile","table_context","type","values"],"concept_alias_group":"updated_at"}],"table_description":"The \"suppliers\" table stores information about suppliers, including their unique identifier, name, contact details, and timestamps for record creation and updates.","glossary_terms":["RetailDomainGlossary.SupplierCode"],"primary_keys":["supplier_id"],"foreign_keys":[],"row_count":10,"field_classifications":{"contact_name":"person_name","email":"contact","phone":"contact","created_at":"temporal","updated_at":"temporal"},"sensitive_fields":{"email":"pii_contact","phone":"pii_contact"},"incremental_columns":["updated_at"],"join_candidates":[],"unit_summary":{"columns_with_units":0,"columns_without_units":7,"mixed_unit_groups":[],"unknown_unit_columns":[]},"cdc_enabled":false,"has_primary_key":true,"has_foreign_keys":false,"has_sensitive_fields":true,"row_count_projection_1y":22,"row_count_projection_2y":35,"row_count_projection_5y":74,"partition_columns_candidates":["created_at","updated_at"],"classification_summary":{"concept_counts":{"contact.email":1,"contact.person_name":2,"contact.phone":1,"identifier.foreign_key":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":["contact_name","name"]},"data_quality":{"findings":[{"column":"email","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 10 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":"phone","check":"nullable_but_never_null","severity":"info","detail":"Column is nullable but has 0 NULLs across 10 row(s)","recommendation":"Consider adding a NOT NULL constraint if the column should always have a value"},{"column":null,"check":"timestamp_ordering","severity":"info","detail":"Table has both 'created_at' and 'updated_at' but no CHECK constraint guaranteeing created_at &lt;= updated_at.","recommendation":"Add CHECK (created_at &lt;= updated_at) to enforce temporal consistency.","created_column":"created_at","updated_column":"updated_at"},{"column":null,"check":"delete_management","severity":"warning","detail":"No soft-delete column detected and CDC is not enabled. Table likely uses hard deletes invisible to incremental ingestion.","recommendation":"Consider: (1) Add soft-delete column, (2) Enable CDC via ALTER TABLE \u2026 REPLICA IDENTITY FULL, or (3) Plan periodic full-load syncs.","delete_strategy":"hard_delete","soft_delete_column":null,"soft_delete_type":null,"has_audit_trail":false},{"column":null,"check":"timezone","severity":"info","detail":"All 2 date/time column(s) are TZ-naive \u2014 stored values are implicitly in server timezone '(UTC) Coordinated Universal Time'.","recommendation":"During ingestion, treat all timestamps as '(UTC) Coordinated Universal Time' and convert to UTC.","server_timezone":"(UTC) Coordinated Universal Time","columns":[{"column":"created_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false},{"column":"updated_at","type":"datetime2","effective_timezone":"(UTC) Coordinated Universal Time","is_tz_aware":false}],"distinct_timezones":["(UTC) Coordinated Universal Time"],"tz_aware_count":0,"tz_naive_count":2}]}}]}</t>
         </is>
       </c>
     </row>
@@ -10416,7 +10512,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>2026-04-03T12:09:52.790221+00:00</t>
+          <t>2026-04-07T08:55:59.245988+00:00</t>
         </is>
       </c>
       <c r="C3" s="4" t="n"/>
@@ -15535,7 +15631,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="41" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -15671,10 +15767,14 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>The `customers` table stores information about retail customers, including their unique ID, name, contact details, and timestamps for record creation and updates.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
+          <t>The "customers" table stores information about retail customers, including their unique ID, name, contact details, and timestamps for record creation and updates.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.CustomerIdentifier</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>{"concept_counts":{"contact.email":1,"contact.person_name":2,"contact.phone":1,"identifier.foreign_key":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":[]}</t>
@@ -16019,7 +16119,11 @@
           <t>Unique identifier for each customer in the retail operations system.</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.CustomerIdentifier</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -16103,7 +16207,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Stores the given name of a customer as a non-null, case-insensitive Unicode string.</t>
+          <t>Stores the given name of a customer as a non-null Unicode string.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -16190,10 +16294,14 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Stores the last name of a customer as a non-null, case-insensitive Unicode string.</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr"/>
+          <t>The "last_name" column in the "customers" table stores the non-nullable family name of a customer as a case-insensitive Unicode string.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.Customer</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>contact.person_name</t>
@@ -16281,7 +16389,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Stores the email address of the customer, allowing null values.</t>
+          <t>Stores the email address of the customer, allowing null values for cases where an email is not provided.</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -16546,7 +16654,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Tracks the timestamp of the most recent update to a customer's record, ensuring accurate change history.</t>
+          <t>Tracks the timestamp of the most recent update to a customer record, ensuring accurate audit and change history.</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -17198,7 +17306,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>The `employees` table stores details about retail system employees, including their identifiers, store associations, personal information, roles, hire dates, and record timestamps.</t>
+          <t>The `employees` table stores detailed information about retail system employees, including their unique identifiers, store assignments, personal details, job roles, hire dates, and record timestamps.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -17651,7 +17759,7 @@
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Unique identifier for each employee in the retail operations system.</t>
+          <t>Unique identifier for employees in the retail operations system.</t>
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
@@ -17730,7 +17838,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Associates each employee with a specific store, referencing the `store_id` column in the `stores` table.</t>
+          <t>Identifies the store where the employee is assigned, referencing the `store_id` column in the `stores` table.</t>
         </is>
       </c>
       <c r="K30" t="inlineStr"/>
@@ -17817,7 +17925,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Stores the given name of an employee, represented as a non-null, case-insensitive Unicode string.</t>
+          <t>Stores the given name of an employee, represented as a non-null Unicode string.</t>
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
@@ -17904,7 +18012,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>The "last_name" column in the "employees" table stores the non-nullable family name of an employee as a case-insensitive Unicode string.</t>
+          <t>The "last_name" column in the "employees" table stores the non-nullable family name of each employee as a case-insensitive Unicode string.</t>
         </is>
       </c>
       <c r="K32" t="inlineStr"/>
@@ -17995,7 +18103,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Stores the unique email address of each employee for contact purposes, with a maximum length of 450 characters and cannot be null.</t>
+          <t>The "email" column in the "employees" table stores the unique, non-null email address of each employee for contact purposes.</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -18074,7 +18182,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Indicates the job position or function of an employee within the organization, stored as a non-nullable text value.</t>
+          <t>Stores the job role or position of an employee within the organization, such as "Cashier" or "Sales," as a non-null text value.</t>
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
@@ -18335,7 +18443,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>The `updated_at` column stores the non-nullable timestamp of the most recent update to an employee record.</t>
+          <t>The `updated_at` column in the `employees` table stores the non-nullable timestamp of the most recent update to an employee record.</t>
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
@@ -18865,7 +18973,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="80" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -19004,7 +19112,11 @@
           <t>Current stock levels with normalized stock unit representation.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.Inventory, RetailDomainGlossary.InventoryByProductAndLocation</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>{"concept_counts":{"identifier.foreign_key":3,"measure.quantity":1,"temporal.created_at":1,"temporal.event_time":1,"temporal.updated_at":1},"low_confidence_columns":["reorder_level","stock_unit"]}</t>
@@ -19567,7 +19679,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Identifier for the store associated with the inventory record, referencing the `store_id` column in the `stores` table.</t>
+          <t>Represents the unique identifier of the store associated with the inventory record, referencing the `store_id` column in the `stores` table.</t>
         </is>
       </c>
       <c r="K32" t="inlineStr"/>
@@ -19650,7 +19762,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>References the unique identifier of a product from the `products` table to associate inventory records with specific products.</t>
+          <t>References the unique identifier of a product from the products table, linking inventory records to specific products.</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -19737,10 +19849,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Tracks the current quantity of a product available in inventory, expressed as a non-null integer.</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
+          <t>The `quantity_on_hand` column in the `inventory` table stores the current stock level of a product as a non-null integer.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.Inventory</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>measure.quantity</t>
@@ -19835,7 +19951,11 @@
           <t>Indicates the minimum quantity of a product in inventory that triggers a reorder, stored as a non-null integer.</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.ReorderPoint</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="n">
         <v>0.1</v>
@@ -19914,7 +20034,11 @@
           <t>The `last_restocked_at` column records the timestamp of the most recent restocking event for an inventory item, allowing null values if the item has not been restocked.</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.Replenishment</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>temporal.event_time</t>
@@ -20164,10 +20288,14 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Represents the monetary value of inventory stock, stored as a numeric value with up to 10 digits and 2 decimal places, and may be null.</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
+          <t>Represents the monetary value of inventory stock, stored as a numeric value with two decimal places, and may be null.</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.Inventory</t>
+        </is>
+      </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="n">
         <v>0</v>
@@ -20230,7 +20358,11 @@
           <t>Current stock unit label.</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.UnitOfMeasure</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="n">
         <v>0.15</v>
@@ -20727,7 +20859,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="67" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -20866,7 +20998,11 @@
           <t>Master product catalog including physical units for analyzer unit-context testing.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.Inventory, RetailDomainGlossary.SupplierCode</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>{"concept_counts":{"contact.person_name":1,"entity.category":1,"finance.currency_amount":2,"identifier.foreign_key":3,"identifier.product_code":1,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":["length_unit","name","product_description","weight_unit"]}</t>
@@ -21344,10 +21480,14 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Unique identifier for each product in the retail operations system.</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr"/>
+          <t>Unique identifier for each product in the retail system, serving as the primary key for the products table.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.Barcode</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -21426,7 +21566,11 @@
           <t>The `supplier_id` column in the `products` table is a non-nullable foreign key referencing the `supplier_id` column in the `suppliers` table, identifying the supplier associated with each product.</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SupplierCode</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -21506,10 +21650,14 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Unique alphanumeric identifier for a product used for inventory and sales tracking, stored as a non-null nvarchar(450).</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr"/>
+          <t>Unique alphanumeric identifier for a product used for inventory and sales tracking.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.Product</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>identifier.product_code</t>
@@ -21585,7 +21733,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>The "name" column in the "products" table stores the non-nullable name of a product as a case-insensitive Unicode string.</t>
+          <t>Stores the name of the product as a non-null, case-insensitive Unicode string.</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -21672,10 +21820,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Indicates the product's category classification, such as "Books," "Clothing," or "Electronics," stored as a non-null, case-insensitive text value.</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
+          <t>Indicates the product's category classification, such as "Books," "Clothing," or "Electronics," stored as a non-nullable nvarchar value.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.ProductCategory</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>entity.category</t>
@@ -21759,10 +21911,14 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Stores the retail price of a product as a non-null numeric value with up to 10 digits and 2 decimal places.</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
+          <t>The `unit_price` column stores the non-null selling price of a product as a numeric value with up to 10 digits and 2 decimal places, representing a currency amount.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SellingPrice</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>finance.currency_amount</t>
@@ -21846,10 +22002,14 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Represents the numeric cost price of a product in the retail system, stored as a non-nullable currency amount with up to 10 digits and 2 decimal places.</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
+          <t>The `cost_price` column stores the non-null numeric cost amount (up to 10 digits with 2 decimal places) representing the purchase price of a product in the retail system.</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.CostPrice</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>finance.currency_amount</t>
@@ -21996,7 +22156,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Indicates the timestamp when the product record was initially created, stored as a non-nullable datetime value.</t>
+          <t>The `created_at` column stores the non-nullable timestamp indicating when a product record was initially created in the system.</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -22169,7 +22329,11 @@
           <t>Source weight unit (kg/lb) used for unit inference testing.</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.UnitOfMeasure</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="n">
         <v>0.15</v>
@@ -22252,7 +22416,11 @@
           <t>The `weight_value` column stores the weight of a product as a numeric value with up to 10 digits and 2 decimal places, and it is nullable.</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.UnitOfMeasure</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="n">
         <v>0</v>
@@ -22332,7 +22500,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>The "length_value" column stores the numeric length measurement of a product, allowing up to 10 digits with 2 decimal places, and is nullable.</t>
+          <t>Represents the length measurement of a product in numeric format, allowing null values.</t>
         </is>
       </c>
       <c r="K42" t="inlineStr"/>
@@ -22418,7 +22586,11 @@
           <t>Source length unit (cm/in) used for unit inference testing.</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.UnitOfMeasure</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="n">
         <v>0.15</v>
@@ -22494,10 +22666,14 @@
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Stores optional textual details about a product, such as features or specifications, with support for Unicode characters.</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr"/>
+          <t>Stores optional textual details about a product, such as features or specifications.</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.Product</t>
+        </is>
+      </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="n">
         <v>0.1</v>
@@ -22560,7 +22736,11 @@
           <t>Primary supplier relationship used for join candidate detection.</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.SupplierPurchaseRelationship</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -23323,7 +23503,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
     <col width="80" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="80" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
@@ -23462,7 +23642,11 @@
           <t>Line items with order quantities and explicit unit labels.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.OrderLine, RetailDomainGlossary.UnitOfMeasure, RetailDomainGlossary.CostPrice, RetailDomainGlossary.PurchaseOrder</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>{"concept_counts":{"finance.currency_amount":1,"identifier.foreign_key":3,"measure.quantity":3,"temporal.created_at":1,"temporal.updated_at":1},"low_confidence_columns":[]}</t>
@@ -23939,7 +24123,11 @@
           <t>Unique identifier for each purchase order item record in the `purchase_order_items` table.</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.OrderLine</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -24015,10 +24203,14 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Links each purchase order item to its corresponding purchase order in the `purchase_orders` table via a non-null foreign key.</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
+          <t>Represents the unique identifier of the associated purchase order, linking purchase order items to their parent purchase order in the `purchase_orders` table.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.PurchaseOrder</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -24101,7 +24293,11 @@
           <t>Identifier linking each purchase order item to a specific product in the products table.</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.ProductCategory</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>identifier.foreign_key</t>
@@ -24188,7 +24384,11 @@
           <t>The `quantity` column in the `purchase_order_items` table stores the non-null integer value representing the number of units of a product included in a specific purchase order item.</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.UnitOfMeasure</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>measure.quantity</t>
@@ -24288,10 +24488,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>The `unit_cost` column in the `purchase_order_items` table stores the non-null numeric cost per unit of a product in a purchase order, represented as a currency amount with up to 10 digits and 2 decimal places.</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
+          <t>Represents the per-unit cost of a product in a purchase order, stored as a non-null numeric value with up to 10 digits and 2 decimal places.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.CostPrice</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>finance.currency_amount</t>
@@ -24375,7 +24579,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Records the timestamp when a purchase order item entry is created, stored as a non-nullable datetime value.</t>
+          <t>The `created_at` column records the non-nullable timestamp indicating when each purchase order item record was created.</t>
         </is>
       </c>
       <c r="K35" t="inlineStr"/>
@@ -24462,7 +24666,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>The `updated_at` column in the `purchase_order_items` table stores the non-nullable timestamp of the most recent update to a purchase order item record.</t>
+          <t>Records the timestamp of the most recent update to a purchase order item, ensuring accurate tracking of modifications.</t>
         </is>
       </c>
       <c r="K36" t="inlineStr"/>
@@ -24552,7 +24756,11 @@
           <t>The `ordered_qty_value` column stores the numeric quantity value (up to two decimal places) of items ordered in a purchase order, which can be null.</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.PurchaseOrder</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>measure.quantity</t>
@@ -24647,7 +24855,11 @@
           <t>Ordered quantity unit (ea/box).</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>RetailDomainGlossary.UnitOfMeasure</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>measure.quantity</t>

</xml_diff>